<commit_message>
docs: pre-fill recommended ranking/triage in the launch+parked workbook
Launch tab: ranks 1-16 doable NOW (pre-build), 17-25 batch at build #35 (~Jul 1),
26 = submit. Parked tab triaged: 7 BEFORE LAUNCH (P-71 rename blocker, targeted
a11y P-28/29, quick CI/error-handling P-23/63/64, light analytics P-73), 2
VERIFY->drop (P-33 hide-balances, P-59 Sentry — likely already shipped), 12 SOON
(v1.1), rest LATER. Columns are recommendations to override.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/finwise-launch-and-parked.xlsx
+++ b/docs/finwise-launch-and-parked.xlsx
@@ -19,12 +19,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="640" uniqueCount="414">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="740" uniqueCount="426">
   <si>
     <t>Launch Checklist</t>
   </si>
   <si>
-    <t>Everything left to ship v1, by phase. 'Type' = Blocker (can't ship without) / Recommended / Optional. Owner: You = account/legal/manual · Claude = in-repo. Statuses reconciled against code/records on 2026-06-26 (a few launch-checklist.md rows were stale — e.g. Firestore rules ARE deployed). Fill the yellow 'Your rank' + 'Decision' columns to set the order we work them. Rows marked 'VERIFY' are doc/memory-derived — confirm in code before relying.</t>
+    <t>Everything left to ship v1, by phase. 'Type' = Blocker (can't ship without) / Recommended / Optional. Owner: You = account/legal/manual · Claude = in-repo. Statuses reconciled against code/records on 2026-06-26 (a few launch-checklist.md rows were stale — e.g. Firestore rules ARE deployed). The yellow 'Your rank' + 'Decision' columns are PRE-FILLED with Claude's recommended order — override freely. Headline: ranks 1-16 can all happen NOW (before the build resets); 17-25 batch at build #35 (~Jul 1); 26 = submit. 'VERIFY' rows are doc/memory-derived — confirm in code before relying.</t>
   </si>
   <si>
     <t>ID</t>
@@ -72,6 +72,9 @@
     <t>OPEN — the long pole</t>
   </si>
   <si>
+    <t>NOW (you+me)</t>
+  </si>
+  <si>
     <t>You pick a vendor + API key (~$10–50/mo EOD); then a ~1-file PriceProvider swap in marketData.ts. Legal blocker.</t>
   </si>
   <si>
@@ -90,6 +93,9 @@
     <t>DONE 2026-06-17 (checklist doc is STALE)</t>
   </si>
   <si>
+    <t>DONE — confirm in console</t>
+  </si>
+  <si>
     <t>Deployed to finwise-app-jj with the privilege-escalation fix + emulator tests. Verify active in console.</t>
   </si>
   <si>
@@ -108,6 +114,9 @@
     <t>BLOCKED on EAS free quota (~Jul 1); code READY</t>
   </si>
   <si>
+    <t>AT BUILD #35</t>
+  </si>
+  <si>
     <t>739 tests green, tsc clean, T22 loop fix in. Push-button once quota resets. eas build --local fails (macOS-26 keychain).</t>
   </si>
   <si>
@@ -135,6 +144,9 @@
     <t>DRAFTED — needs entry</t>
   </si>
   <si>
+    <t>NOW (you)</t>
+  </si>
+  <si>
     <t>Copy ready in finwise-appstore-listing.md; paste into App Store Connect.</t>
   </si>
   <si>
@@ -240,6 +252,9 @@
     <t>DONE (bb68bad)</t>
   </si>
   <si>
+    <t>DONE</t>
+  </si>
+  <si>
     <t>Shared &lt;Disclaimer/&gt; on all judgment screens; coverage guard test.</t>
   </si>
   <si>
@@ -267,6 +282,9 @@
     <t>LIKELY DONE on taxonomy-v1.0.7 — VERIFY</t>
   </si>
   <si>
+    <t>NOW — verify (me)</t>
+  </si>
+  <si>
     <t>take_home_agreement.test + number_agreement.test pass. Confirm the % path specifically.</t>
   </si>
   <si>
@@ -330,6 +348,9 @@
     <t>DECISION — likely already (USD-only, picker removed)</t>
   </si>
   <si>
+    <t>NOW — decide</t>
+  </si>
+  <si>
     <t>Confirm; don't market global. GLBA/state-privacy posture assumes US.</t>
   </si>
   <si>
@@ -390,13 +411,16 @@
     <t>Final step</t>
   </si>
   <si>
+    <t>SUBMIT (last)</t>
+  </si>
+  <si>
     <t>eas submit is separate from the build quota.</t>
   </si>
   <si>
     <t>Parked - Backlog</t>
   </si>
   <si>
-    <t>Every consciously-deferred item, deduplicated across all docs (features, roadmap, qa-plan, ui-compliance, scorecard, microservices, onboarding-matrix, rename-candidates). Status: Open / Partial / Done-verify (doc says open but code/memory says shipped — verify &amp; drop) / Decision. Fill the yellow 'Your rank' + 'Decision' (do-now / next / later / drop) columns. Source = which doc(s) it came from.</t>
+    <t>Every consciously-deferred item, deduplicated across all docs (features, roadmap, qa-plan, ui-compliance, scorecard, microservices, onboarding-matrix, rename-candidates). Status: Open / Partial / Done-verify (doc says open but code/memory says shipped — verify &amp; drop). The yellow 'Your rank' + 'Decision' columns are PRE-FILLED with Claude's recommended triage — override freely. Recommendation: only 7 items 'BEFORE LAUNCH' (P-71 rename is a real blocker; targeted a11y; quick CI/error-handling; light analytics), 2 to VERIFY → drop, 12 'SOON (v1.1)', the rest 'LATER'. Source = which doc(s) it came from.</t>
   </si>
   <si>
     <t>Category</t>
@@ -426,6 +450,9 @@
     <t>features, roadmap, scorecard, microservices</t>
   </si>
   <si>
+    <t>LATER (v1.x / v2)</t>
+  </si>
+  <si>
     <t>Auto-pull balances/transactions behind an aggregator interface. XL effort, server-side (Cloud Functions). Biggest stickiness/friction lever.</t>
   </si>
   <si>
@@ -459,6 +486,9 @@
     <t>features, roadmap</t>
   </si>
   <si>
+    <t>SOON (v1.1)</t>
+  </si>
+  <si>
     <t>npx expo run:ios native rebuild, then test a real scan. Launch-adjacent — folds into build #35.</t>
   </si>
   <si>
@@ -675,6 +705,9 @@
     <t>features, qa-plan (T2-005/003)</t>
   </si>
   <si>
+    <t>BEFORE LAUNCH</t>
+  </si>
+  <si>
     <t>Mostly build-time tooling. Add npm audit --audit-level=high + gitleaks to CI.</t>
   </si>
   <si>
@@ -802,6 +835,9 @@
   </si>
   <si>
     <t>features, qa-plan, ui-compliance (G-16)</t>
+  </si>
+  <si>
+    <t>VERIFY → drop</t>
   </si>
   <si>
     <t>features.md says a 'hide-balances mask-ALL' shipped in build #34 — VERIFY in code; likely closable.</t>
@@ -1727,7 +1763,7 @@
     <col min="5" max="5" width="12.7109375" customWidth="1"/>
     <col min="6" max="6" width="30.7109375" customWidth="1"/>
     <col min="7" max="7" width="9.7109375" customWidth="1"/>
-    <col min="8" max="8" width="12.7109375" customWidth="1"/>
+    <col min="8" max="8" width="16.7109375" customWidth="1"/>
     <col min="9" max="9" width="50.7109375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1816,629 +1852,733 @@
       <c r="F5" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="G5" s="6"/>
-      <c r="H5" s="6"/>
+      <c r="G5" s="6">
+        <v>1</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>17</v>
+      </c>
       <c r="I5" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G6" s="6"/>
-      <c r="H6" s="6"/>
+        <v>23</v>
+      </c>
+      <c r="G6" s="6">
+        <v>5</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>24</v>
+      </c>
       <c r="I6" s="4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:9">
       <c r="A7" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E7" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="G7" s="6"/>
-      <c r="H7" s="6"/>
+        <v>30</v>
+      </c>
+      <c r="G7" s="6">
+        <v>17</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>31</v>
+      </c>
       <c r="I7" s="4" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" spans="1:9">
       <c r="A8" s="4" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="G8" s="6"/>
-      <c r="H8" s="6"/>
+        <v>36</v>
+      </c>
+      <c r="G8" s="6">
+        <v>25</v>
+      </c>
+      <c r="H8" s="6" t="s">
+        <v>31</v>
+      </c>
       <c r="I8" s="4" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="9" spans="1:9">
       <c r="A9" s="4" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="G9" s="6"/>
-      <c r="H9" s="6"/>
+        <v>40</v>
+      </c>
+      <c r="G9" s="6">
+        <v>7</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>41</v>
+      </c>
       <c r="I9" s="4" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10" spans="1:9">
       <c r="A10" s="4" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E10" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F10" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="G10" s="6">
+        <v>9</v>
+      </c>
+      <c r="H10" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
       <c r="I10" s="4" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
     </row>
     <row r="11" spans="1:9">
       <c r="A11" s="4" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E11" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
+        <v>49</v>
+      </c>
+      <c r="G11" s="6">
+        <v>11</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>41</v>
+      </c>
       <c r="I11" s="4" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12" spans="1:9">
       <c r="A12" s="4" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E12" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
+        <v>54</v>
+      </c>
+      <c r="G12" s="6">
+        <v>8</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>41</v>
+      </c>
       <c r="I12" s="4" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
     </row>
     <row r="13" spans="1:9">
       <c r="A13" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B13" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="B13" s="4" t="s">
-        <v>48</v>
-      </c>
       <c r="C13" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="G13" s="6"/>
-      <c r="H13" s="6"/>
+        <v>54</v>
+      </c>
+      <c r="G13" s="6">
+        <v>10</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>41</v>
+      </c>
       <c r="I13" s="4" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="14" spans="1:9">
       <c r="A14" s="4" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E14" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="G14" s="6"/>
-      <c r="H14" s="6"/>
+        <v>61</v>
+      </c>
+      <c r="G14" s="6">
+        <v>20</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>31</v>
+      </c>
       <c r="I14" s="4" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
     </row>
     <row r="15" spans="1:9">
       <c r="A15" s="4" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E15" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="G15" s="6"/>
-      <c r="H15" s="6"/>
+        <v>66</v>
+      </c>
+      <c r="G15" s="6">
+        <v>12</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>17</v>
+      </c>
       <c r="I15" s="4" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="16" spans="1:9">
       <c r="A16" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B16" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="B16" s="4" t="s">
-        <v>60</v>
-      </c>
       <c r="C16" s="4" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E16" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="G16" s="6"/>
-      <c r="H16" s="6"/>
+        <v>70</v>
+      </c>
+      <c r="G16" s="6">
+        <v>19</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>31</v>
+      </c>
       <c r="I16" s="4" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
     </row>
     <row r="17" spans="1:9">
       <c r="A17" s="4" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="G17" s="6"/>
-      <c r="H17" s="6"/>
+        <v>76</v>
+      </c>
+      <c r="G17" s="6">
+        <v>15</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>77</v>
+      </c>
       <c r="I17" s="4" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
     </row>
     <row r="18" spans="1:9">
       <c r="A18" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="D18" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="B18" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="C18" s="4" t="s">
+      <c r="E18" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="D18" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>71</v>
-      </c>
       <c r="F18" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="G18" s="6"/>
-      <c r="H18" s="6"/>
+        <v>81</v>
+      </c>
+      <c r="G18" s="6">
+        <v>16</v>
+      </c>
+      <c r="H18" s="6" t="s">
+        <v>77</v>
+      </c>
       <c r="I18" s="4" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
     </row>
     <row r="19" spans="1:9">
       <c r="A19" s="4" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="G19" s="6"/>
-      <c r="H19" s="6"/>
+        <v>86</v>
+      </c>
+      <c r="G19" s="6">
+        <v>2</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>87</v>
+      </c>
       <c r="I19" s="4" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
     </row>
     <row r="20" spans="1:9">
       <c r="A20" s="4" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="G20" s="6"/>
-      <c r="H20" s="6"/>
+        <v>91</v>
+      </c>
+      <c r="G20" s="6">
+        <v>3</v>
+      </c>
+      <c r="H20" s="6" t="s">
+        <v>87</v>
+      </c>
       <c r="I20" s="4" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
     </row>
     <row r="21" spans="1:9">
       <c r="A21" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="G21" s="6">
+        <v>4</v>
+      </c>
+      <c r="H21" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="B21" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="E21" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="F21" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="G21" s="6"/>
-      <c r="H21" s="6"/>
       <c r="I21" s="4" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
     </row>
     <row r="22" spans="1:9">
       <c r="A22" s="4" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="G22" s="6"/>
-      <c r="H22" s="6"/>
+        <v>99</v>
+      </c>
+      <c r="G22" s="6">
+        <v>23</v>
+      </c>
+      <c r="H22" s="6" t="s">
+        <v>31</v>
+      </c>
       <c r="I22" s="4" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
     </row>
     <row r="23" spans="1:9">
       <c r="A23" s="4" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="G23" s="6"/>
-      <c r="H23" s="6"/>
+        <v>103</v>
+      </c>
+      <c r="G23" s="6">
+        <v>6</v>
+      </c>
+      <c r="H23" s="6" t="s">
+        <v>41</v>
+      </c>
       <c r="I23" s="4" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
     </row>
     <row r="24" spans="1:9">
       <c r="A24" s="4" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="G24" s="6"/>
-      <c r="H24" s="6"/>
+        <v>108</v>
+      </c>
+      <c r="G24" s="6">
+        <v>13</v>
+      </c>
+      <c r="H24" s="6" t="s">
+        <v>109</v>
+      </c>
       <c r="I24" s="4" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
     </row>
     <row r="25" spans="1:9">
       <c r="A25" s="4" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="F25" s="9" t="s">
-        <v>106</v>
-      </c>
-      <c r="G25" s="6"/>
-      <c r="H25" s="6"/>
+        <v>113</v>
+      </c>
+      <c r="G25" s="6">
+        <v>14</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>109</v>
+      </c>
       <c r="I25" s="4" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
     </row>
     <row r="26" spans="1:9">
       <c r="A26" s="4" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E26" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="G26" s="6"/>
-      <c r="H26" s="6"/>
+        <v>61</v>
+      </c>
+      <c r="G26" s="6">
+        <v>21</v>
+      </c>
+      <c r="H26" s="6" t="s">
+        <v>31</v>
+      </c>
       <c r="I26" s="4" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
     </row>
     <row r="27" spans="1:9">
       <c r="A27" s="4" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E27" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="G27" s="6"/>
-      <c r="H27" s="6"/>
+        <v>121</v>
+      </c>
+      <c r="G27" s="6">
+        <v>18</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>31</v>
+      </c>
       <c r="I27" s="4"/>
     </row>
     <row r="28" spans="1:9">
       <c r="A28" s="4" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E28" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="G28" s="6"/>
-      <c r="H28" s="6"/>
+        <v>54</v>
+      </c>
+      <c r="G28" s="6">
+        <v>22</v>
+      </c>
+      <c r="H28" s="6" t="s">
+        <v>31</v>
+      </c>
       <c r="I28" s="4"/>
     </row>
     <row r="29" spans="1:9">
       <c r="A29" s="4" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="G29" s="6"/>
-      <c r="H29" s="6"/>
+        <v>99</v>
+      </c>
+      <c r="G29" s="6">
+        <v>24</v>
+      </c>
+      <c r="H29" s="6" t="s">
+        <v>31</v>
+      </c>
       <c r="I29" s="4"/>
     </row>
     <row r="30" spans="1:9">
       <c r="A30" s="4" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E30" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="G30" s="6"/>
-      <c r="H30" s="6"/>
+        <v>129</v>
+      </c>
+      <c r="G30" s="6">
+        <v>26</v>
+      </c>
+      <c r="H30" s="6" t="s">
+        <v>130</v>
+      </c>
       <c r="I30" s="4" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
     </row>
   </sheetData>
@@ -2465,13 +2605,13 @@
     <col min="4" max="4" width="11.7109375" customWidth="1"/>
     <col min="5" max="5" width="26.7109375" customWidth="1"/>
     <col min="6" max="6" width="9.7109375" customWidth="1"/>
-    <col min="7" max="7" width="11.7109375" customWidth="1"/>
+    <col min="7" max="7" width="16.7109375" customWidth="1"/>
     <col min="8" max="8" width="56.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2483,7 +2623,7 @@
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2508,16 +2648,16 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>4</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>8</v>
@@ -2526,1627 +2666,1813 @@
         <v>9</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" s="4" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
+      <c r="G5" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H5" s="4" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" s="4" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="F6" s="6"/>
-      <c r="G6" s="6"/>
+      <c r="G6" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H6" s="4" t="s">
-        <v>139</v>
+        <v>148</v>
       </c>
     </row>
     <row r="7" spans="1:8">
       <c r="A7" s="4" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
+      <c r="G7" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H7" s="4" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" s="4" t="s">
-        <v>143</v>
+        <v>152</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="F8" s="6"/>
-      <c r="G8" s="6"/>
+        <v>154</v>
+      </c>
+      <c r="F8" s="6">
+        <v>8</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>155</v>
+      </c>
       <c r="H8" s="4" t="s">
-        <v>146</v>
+        <v>156</v>
       </c>
     </row>
     <row r="9" spans="1:8">
       <c r="A9" s="4" t="s">
-        <v>147</v>
+        <v>157</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>148</v>
+        <v>158</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
+        <v>159</v>
+      </c>
+      <c r="F9" s="6">
+        <v>12</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>155</v>
+      </c>
       <c r="H9" s="4" t="s">
-        <v>150</v>
+        <v>160</v>
       </c>
     </row>
     <row r="10" spans="1:8">
       <c r="A10" s="4" t="s">
-        <v>151</v>
+        <v>161</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>152</v>
+        <v>162</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>153</v>
+        <v>163</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>154</v>
+        <v>164</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>155</v>
+        <v>165</v>
       </c>
       <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
+      <c r="G10" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H10" s="4" t="s">
-        <v>156</v>
+        <v>166</v>
       </c>
     </row>
     <row r="11" spans="1:8">
       <c r="A11" s="4" t="s">
-        <v>157</v>
+        <v>167</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>152</v>
+        <v>162</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>158</v>
+        <v>168</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
+      <c r="G11" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H11" s="4" t="s">
-        <v>160</v>
+        <v>170</v>
       </c>
     </row>
     <row r="12" spans="1:8">
       <c r="A12" s="4" t="s">
-        <v>161</v>
+        <v>171</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>152</v>
+        <v>162</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>162</v>
+        <v>172</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>163</v>
+        <v>173</v>
       </c>
       <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
+      <c r="G12" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H12" s="4" t="s">
-        <v>164</v>
+        <v>174</v>
       </c>
     </row>
     <row r="13" spans="1:8">
       <c r="A13" s="4" t="s">
-        <v>165</v>
+        <v>175</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>152</v>
+        <v>162</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>166</v>
+        <v>176</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>163</v>
+        <v>173</v>
       </c>
       <c r="F13" s="6"/>
-      <c r="G13" s="6"/>
+      <c r="G13" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H13" s="4"/>
     </row>
     <row r="14" spans="1:8">
       <c r="A14" s="4" t="s">
-        <v>167</v>
+        <v>177</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>169</v>
+        <v>179</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>154</v>
+        <v>164</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="F14" s="6"/>
-      <c r="G14" s="6"/>
+      <c r="G14" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H14" s="4" t="s">
-        <v>171</v>
+        <v>181</v>
       </c>
     </row>
     <row r="15" spans="1:8">
       <c r="A15" s="4" t="s">
-        <v>172</v>
+        <v>182</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>173</v>
+        <v>183</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
+      <c r="G15" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H15" s="4" t="s">
-        <v>174</v>
+        <v>184</v>
       </c>
     </row>
     <row r="16" spans="1:8">
       <c r="A16" s="4" t="s">
-        <v>175</v>
+        <v>185</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>176</v>
+        <v>186</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="F16" s="6"/>
-      <c r="G16" s="6"/>
+      <c r="G16" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H16" s="4"/>
     </row>
     <row r="17" spans="1:8">
       <c r="A17" s="4" t="s">
-        <v>177</v>
+        <v>187</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>178</v>
+        <v>188</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
       <c r="F17" s="6"/>
-      <c r="G17" s="6"/>
+      <c r="G17" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H17" s="4" t="s">
-        <v>180</v>
+        <v>190</v>
       </c>
     </row>
     <row r="18" spans="1:8">
       <c r="A18" s="4" t="s">
-        <v>181</v>
+        <v>191</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>182</v>
+        <v>192</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>183</v>
+        <v>193</v>
       </c>
       <c r="F18" s="6"/>
-      <c r="G18" s="6"/>
+      <c r="G18" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H18" s="4" t="s">
-        <v>184</v>
+        <v>194</v>
       </c>
     </row>
     <row r="19" spans="1:8">
       <c r="A19" s="4" t="s">
-        <v>185</v>
+        <v>195</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>186</v>
+        <v>196</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="F19" s="6"/>
-      <c r="G19" s="6"/>
+      <c r="G19" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H19" s="4" t="s">
-        <v>187</v>
+        <v>197</v>
       </c>
     </row>
     <row r="20" spans="1:8">
       <c r="A20" s="4" t="s">
-        <v>188</v>
+        <v>198</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>189</v>
+        <v>199</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="F20" s="6"/>
-      <c r="G20" s="6"/>
+      <c r="G20" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H20" s="4" t="s">
-        <v>187</v>
+        <v>197</v>
       </c>
     </row>
     <row r="21" spans="1:8">
       <c r="A21" s="4" t="s">
-        <v>190</v>
+        <v>200</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>191</v>
+        <v>201</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="F21" s="6"/>
-      <c r="G21" s="6"/>
+      <c r="G21" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H21" s="4" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
     </row>
     <row r="22" spans="1:8">
       <c r="A22" s="4" t="s">
-        <v>194</v>
+        <v>204</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>196</v>
+        <v>206</v>
       </c>
       <c r="F22" s="6"/>
-      <c r="G22" s="6"/>
+      <c r="G22" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H22" s="4" t="s">
-        <v>197</v>
+        <v>207</v>
       </c>
     </row>
     <row r="23" spans="1:8">
       <c r="A23" s="4" t="s">
-        <v>198</v>
+        <v>208</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>199</v>
+        <v>209</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="F23" s="6"/>
-      <c r="G23" s="6"/>
+      <c r="G23" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H23" s="4" t="s">
-        <v>201</v>
+        <v>211</v>
       </c>
     </row>
     <row r="24" spans="1:8">
       <c r="A24" s="4" t="s">
-        <v>202</v>
+        <v>212</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>203</v>
+        <v>213</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>204</v>
+        <v>214</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>154</v>
+        <v>164</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>205</v>
+        <v>215</v>
       </c>
       <c r="F24" s="6"/>
-      <c r="G24" s="6"/>
+      <c r="G24" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H24" s="4" t="s">
-        <v>206</v>
+        <v>216</v>
       </c>
     </row>
     <row r="25" spans="1:8">
       <c r="A25" s="4" t="s">
-        <v>207</v>
+        <v>217</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>208</v>
+        <v>218</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>209</v>
+        <v>219</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="F25" s="6"/>
-      <c r="G25" s="6"/>
+      <c r="G25" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H25" s="4" t="s">
-        <v>210</v>
+        <v>220</v>
       </c>
     </row>
     <row r="26" spans="1:8">
       <c r="A26" s="4" t="s">
-        <v>211</v>
+        <v>221</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>208</v>
+        <v>218</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>212</v>
+        <v>222</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>213</v>
+        <v>223</v>
       </c>
       <c r="F26" s="6"/>
-      <c r="G26" s="6"/>
+      <c r="G26" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H26" s="4" t="s">
-        <v>214</v>
+        <v>224</v>
       </c>
     </row>
     <row r="27" spans="1:8">
       <c r="A27" s="4" t="s">
-        <v>215</v>
+        <v>225</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>208</v>
+        <v>218</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>216</v>
+        <v>226</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="F27" s="6"/>
-      <c r="G27" s="6"/>
+        <v>227</v>
+      </c>
+      <c r="F27" s="6">
+        <v>2</v>
+      </c>
+      <c r="G27" s="6" t="s">
+        <v>228</v>
+      </c>
       <c r="H27" s="4" t="s">
-        <v>218</v>
+        <v>229</v>
       </c>
     </row>
     <row r="28" spans="1:8">
       <c r="A28" s="4" t="s">
-        <v>219</v>
+        <v>230</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>208</v>
+        <v>218</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>220</v>
+        <v>231</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>221</v>
+        <v>232</v>
       </c>
       <c r="F28" s="6"/>
-      <c r="G28" s="6"/>
+      <c r="G28" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H28" s="4" t="s">
-        <v>222</v>
+        <v>233</v>
       </c>
     </row>
     <row r="29" spans="1:8">
       <c r="A29" s="4" t="s">
-        <v>223</v>
+        <v>234</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>208</v>
+        <v>218</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>224</v>
+        <v>235</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>225</v>
+        <v>236</v>
       </c>
       <c r="F29" s="6"/>
-      <c r="G29" s="6"/>
+      <c r="G29" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H29" s="4" t="s">
-        <v>226</v>
+        <v>237</v>
       </c>
     </row>
     <row r="30" spans="1:8">
       <c r="A30" s="4" t="s">
-        <v>227</v>
+        <v>238</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>208</v>
+        <v>218</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>228</v>
+        <v>239</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>229</v>
+        <v>240</v>
       </c>
       <c r="F30" s="6"/>
-      <c r="G30" s="6"/>
+      <c r="G30" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H30" s="4" t="s">
-        <v>230</v>
+        <v>241</v>
       </c>
     </row>
     <row r="31" spans="1:8">
       <c r="A31" s="4" t="s">
-        <v>231</v>
+        <v>242</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>208</v>
+        <v>218</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>232</v>
+        <v>243</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>233</v>
+        <v>244</v>
       </c>
       <c r="F31" s="6"/>
-      <c r="G31" s="6"/>
+      <c r="G31" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H31" s="4" t="s">
-        <v>234</v>
+        <v>245</v>
       </c>
     </row>
     <row r="32" spans="1:8">
       <c r="A32" s="4" t="s">
-        <v>235</v>
+        <v>246</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>236</v>
+        <v>247</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>237</v>
+        <v>248</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>238</v>
-      </c>
-      <c r="F32" s="6"/>
-      <c r="G32" s="6"/>
+        <v>249</v>
+      </c>
+      <c r="F32" s="6">
+        <v>3</v>
+      </c>
+      <c r="G32" s="6" t="s">
+        <v>228</v>
+      </c>
       <c r="H32" s="4" t="s">
-        <v>239</v>
+        <v>250</v>
       </c>
     </row>
     <row r="33" spans="1:8">
       <c r="A33" s="4" t="s">
-        <v>240</v>
+        <v>251</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>236</v>
+        <v>247</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>241</v>
+        <v>252</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>242</v>
-      </c>
-      <c r="F33" s="6"/>
-      <c r="G33" s="6"/>
+        <v>253</v>
+      </c>
+      <c r="F33" s="6">
+        <v>4</v>
+      </c>
+      <c r="G33" s="6" t="s">
+        <v>228</v>
+      </c>
       <c r="H33" s="4" t="s">
-        <v>243</v>
+        <v>254</v>
       </c>
     </row>
     <row r="34" spans="1:8">
       <c r="A34" s="4" t="s">
-        <v>244</v>
+        <v>255</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>236</v>
+        <v>247</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>245</v>
+        <v>256</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>246</v>
+        <v>257</v>
       </c>
       <c r="F34" s="6"/>
-      <c r="G34" s="6"/>
+      <c r="G34" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H34" s="4" t="s">
-        <v>247</v>
+        <v>258</v>
       </c>
     </row>
     <row r="35" spans="1:8">
       <c r="A35" s="4" t="s">
-        <v>248</v>
+        <v>259</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>236</v>
+        <v>247</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>249</v>
+        <v>260</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>250</v>
+        <v>261</v>
       </c>
       <c r="F35" s="6"/>
-      <c r="G35" s="6"/>
+      <c r="G35" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H35" s="4" t="s">
-        <v>251</v>
+        <v>262</v>
       </c>
     </row>
     <row r="36" spans="1:8">
       <c r="A36" s="4" t="s">
-        <v>252</v>
+        <v>263</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>236</v>
+        <v>247</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>253</v>
+        <v>264</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>254</v>
+        <v>265</v>
       </c>
       <c r="F36" s="6"/>
-      <c r="G36" s="6"/>
+      <c r="G36" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H36" s="4" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
     </row>
     <row r="37" spans="1:8">
       <c r="A37" s="4" t="s">
-        <v>256</v>
+        <v>267</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>257</v>
+        <v>268</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>258</v>
+        <v>269</v>
       </c>
       <c r="D37" s="8" t="s">
-        <v>259</v>
+        <v>270</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>260</v>
+        <v>271</v>
       </c>
       <c r="F37" s="6"/>
-      <c r="G37" s="6"/>
+      <c r="G37" s="6" t="s">
+        <v>272</v>
+      </c>
       <c r="H37" s="4" t="s">
-        <v>261</v>
+        <v>273</v>
       </c>
     </row>
     <row r="38" spans="1:8">
       <c r="A38" s="4" t="s">
-        <v>262</v>
+        <v>274</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>257</v>
+        <v>268</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>263</v>
+        <v>275</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="F38" s="6"/>
-      <c r="G38" s="6"/>
+        <v>154</v>
+      </c>
+      <c r="F38" s="6">
+        <v>17</v>
+      </c>
+      <c r="G38" s="6" t="s">
+        <v>155</v>
+      </c>
       <c r="H38" s="4" t="s">
-        <v>264</v>
+        <v>276</v>
       </c>
     </row>
     <row r="39" spans="1:8">
       <c r="A39" s="4" t="s">
-        <v>265</v>
+        <v>277</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>257</v>
+        <v>268</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>266</v>
+        <v>278</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="F39" s="6"/>
-      <c r="G39" s="6"/>
+        <v>147</v>
+      </c>
+      <c r="F39" s="6">
+        <v>18</v>
+      </c>
+      <c r="G39" s="6" t="s">
+        <v>155</v>
+      </c>
       <c r="H39" s="4" t="s">
-        <v>267</v>
+        <v>279</v>
       </c>
     </row>
     <row r="40" spans="1:8">
       <c r="A40" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="B40" s="4" t="s">
         <v>268</v>
       </c>
-      <c r="B40" s="4" t="s">
-        <v>257</v>
-      </c>
       <c r="C40" s="4" t="s">
-        <v>269</v>
+        <v>281</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>154</v>
+        <v>164</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="F40" s="6"/>
-      <c r="G40" s="6"/>
+      <c r="G40" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H40" s="4" t="s">
-        <v>270</v>
+        <v>282</v>
       </c>
     </row>
     <row r="41" spans="1:8">
       <c r="A41" s="4" t="s">
-        <v>271</v>
+        <v>283</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>257</v>
+        <v>268</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>272</v>
+        <v>284</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>273</v>
+        <v>285</v>
       </c>
       <c r="F41" s="6"/>
-      <c r="G41" s="6"/>
+      <c r="G41" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H41" s="4" t="s">
-        <v>274</v>
+        <v>286</v>
       </c>
     </row>
     <row r="42" spans="1:8">
       <c r="A42" s="4" t="s">
-        <v>275</v>
+        <v>287</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>257</v>
+        <v>268</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>276</v>
+        <v>288</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="F42" s="6"/>
-      <c r="G42" s="6"/>
+        <v>147</v>
+      </c>
+      <c r="F42" s="6">
+        <v>10</v>
+      </c>
+      <c r="G42" s="6" t="s">
+        <v>155</v>
+      </c>
       <c r="H42" s="4" t="s">
-        <v>277</v>
+        <v>289</v>
       </c>
     </row>
     <row r="43" spans="1:8">
       <c r="A43" s="4" t="s">
-        <v>278</v>
+        <v>290</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>257</v>
+        <v>268</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>279</v>
+        <v>291</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>280</v>
-      </c>
-      <c r="F43" s="6"/>
-      <c r="G43" s="6"/>
+        <v>292</v>
+      </c>
+      <c r="F43" s="6">
+        <v>13</v>
+      </c>
+      <c r="G43" s="6" t="s">
+        <v>155</v>
+      </c>
       <c r="H43" s="4" t="s">
-        <v>281</v>
+        <v>293</v>
       </c>
     </row>
     <row r="44" spans="1:8">
       <c r="A44" s="4" t="s">
-        <v>282</v>
+        <v>294</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>257</v>
+        <v>268</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>283</v>
+        <v>295</v>
       </c>
       <c r="D44" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E44" s="4" t="s">
-        <v>284</v>
+        <v>296</v>
       </c>
       <c r="F44" s="6"/>
-      <c r="G44" s="6"/>
+      <c r="G44" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H44" s="4" t="s">
-        <v>285</v>
+        <v>297</v>
       </c>
     </row>
     <row r="45" spans="1:8">
       <c r="A45" s="4" t="s">
-        <v>286</v>
+        <v>298</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>257</v>
+        <v>268</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>287</v>
+        <v>299</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E45" s="4" t="s">
-        <v>288</v>
-      </c>
-      <c r="F45" s="6"/>
-      <c r="G45" s="6"/>
+        <v>300</v>
+      </c>
+      <c r="F45" s="6">
+        <v>14</v>
+      </c>
+      <c r="G45" s="6" t="s">
+        <v>155</v>
+      </c>
       <c r="H45" s="4" t="s">
-        <v>289</v>
+        <v>301</v>
       </c>
     </row>
     <row r="46" spans="1:8">
       <c r="A46" s="4" t="s">
-        <v>290</v>
+        <v>302</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>257</v>
+        <v>268</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>291</v>
+        <v>303</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>154</v>
+        <v>164</v>
       </c>
       <c r="E46" s="4" t="s">
-        <v>292</v>
-      </c>
-      <c r="F46" s="6"/>
-      <c r="G46" s="6"/>
+        <v>304</v>
+      </c>
+      <c r="F46" s="6">
+        <v>16</v>
+      </c>
+      <c r="G46" s="6" t="s">
+        <v>155</v>
+      </c>
       <c r="H46" s="4" t="s">
-        <v>293</v>
+        <v>305</v>
       </c>
     </row>
     <row r="47" spans="1:8">
       <c r="A47" s="4" t="s">
-        <v>294</v>
+        <v>306</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>257</v>
+        <v>268</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>295</v>
+        <v>307</v>
       </c>
       <c r="D47" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E47" s="4" t="s">
-        <v>296</v>
+        <v>308</v>
       </c>
       <c r="F47" s="6"/>
-      <c r="G47" s="6"/>
+      <c r="G47" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H47" s="4" t="s">
-        <v>297</v>
+        <v>309</v>
       </c>
     </row>
     <row r="48" spans="1:8">
       <c r="A48" s="4" t="s">
-        <v>298</v>
+        <v>310</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>257</v>
+        <v>268</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>299</v>
+        <v>311</v>
       </c>
       <c r="D48" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E48" s="4" t="s">
-        <v>300</v>
+        <v>312</v>
       </c>
       <c r="F48" s="6"/>
-      <c r="G48" s="6"/>
+      <c r="G48" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H48" s="4" t="s">
-        <v>301</v>
+        <v>313</v>
       </c>
     </row>
     <row r="49" spans="1:8">
       <c r="A49" s="4" t="s">
-        <v>302</v>
+        <v>314</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>257</v>
+        <v>268</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>303</v>
+        <v>315</v>
       </c>
       <c r="D49" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E49" s="4" t="s">
-        <v>304</v>
+        <v>316</v>
       </c>
       <c r="F49" s="6"/>
-      <c r="G49" s="6"/>
+      <c r="G49" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H49" s="4" t="s">
-        <v>305</v>
+        <v>317</v>
       </c>
     </row>
     <row r="50" spans="1:8">
       <c r="A50" s="4" t="s">
-        <v>306</v>
+        <v>318</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>257</v>
+        <v>268</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>307</v>
+        <v>319</v>
       </c>
       <c r="D50" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>308</v>
+        <v>320</v>
       </c>
       <c r="F50" s="6"/>
-      <c r="G50" s="6"/>
+      <c r="G50" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H50" s="4" t="s">
-        <v>309</v>
+        <v>321</v>
       </c>
     </row>
     <row r="51" spans="1:8">
       <c r="A51" s="4" t="s">
-        <v>310</v>
+        <v>322</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>257</v>
+        <v>268</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>311</v>
+        <v>323</v>
       </c>
       <c r="D51" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>312</v>
+        <v>324</v>
       </c>
       <c r="F51" s="6"/>
-      <c r="G51" s="6"/>
+      <c r="G51" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H51" s="4" t="s">
-        <v>313</v>
+        <v>325</v>
       </c>
     </row>
     <row r="52" spans="1:8">
       <c r="A52" s="4" t="s">
-        <v>314</v>
+        <v>326</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>257</v>
+        <v>268</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>315</v>
+        <v>327</v>
       </c>
       <c r="D52" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E52" s="4" t="s">
-        <v>316</v>
+        <v>328</v>
       </c>
       <c r="F52" s="6"/>
-      <c r="G52" s="6"/>
+      <c r="G52" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H52" s="4" t="s">
-        <v>317</v>
+        <v>329</v>
       </c>
     </row>
     <row r="53" spans="1:8">
       <c r="A53" s="4" t="s">
-        <v>318</v>
+        <v>330</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>257</v>
+        <v>268</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>319</v>
+        <v>331</v>
       </c>
       <c r="D53" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>320</v>
+        <v>332</v>
       </c>
       <c r="F53" s="6"/>
-      <c r="G53" s="6"/>
+      <c r="G53" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H53" s="4" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
     </row>
     <row r="54" spans="1:8">
       <c r="A54" s="4" t="s">
-        <v>321</v>
+        <v>333</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>257</v>
+        <v>268</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>322</v>
+        <v>334</v>
       </c>
       <c r="D54" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E54" s="4" t="s">
-        <v>323</v>
+        <v>335</v>
       </c>
       <c r="F54" s="6"/>
-      <c r="G54" s="6"/>
+      <c r="G54" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H54" s="4" t="s">
-        <v>324</v>
+        <v>336</v>
       </c>
     </row>
     <row r="55" spans="1:8">
       <c r="A55" s="4" t="s">
-        <v>325</v>
+        <v>337</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>257</v>
+        <v>268</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>326</v>
+        <v>338</v>
       </c>
       <c r="D55" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E55" s="4" t="s">
-        <v>327</v>
+        <v>339</v>
       </c>
       <c r="F55" s="6"/>
-      <c r="G55" s="6"/>
+      <c r="G55" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H55" s="4" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
     </row>
     <row r="56" spans="1:8">
       <c r="A56" s="4" t="s">
-        <v>328</v>
+        <v>340</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>329</v>
+        <v>341</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>330</v>
+        <v>342</v>
       </c>
       <c r="D56" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E56" s="4" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="F56" s="6"/>
-      <c r="G56" s="6"/>
+      <c r="G56" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H56" s="4" t="s">
-        <v>331</v>
+        <v>343</v>
       </c>
     </row>
     <row r="57" spans="1:8">
       <c r="A57" s="4" t="s">
-        <v>332</v>
+        <v>344</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>329</v>
+        <v>341</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>333</v>
+        <v>345</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>154</v>
+        <v>164</v>
       </c>
       <c r="E57" s="4" t="s">
-        <v>273</v>
-      </c>
-      <c r="F57" s="6"/>
-      <c r="G57" s="6"/>
+        <v>285</v>
+      </c>
+      <c r="F57" s="6">
+        <v>11</v>
+      </c>
+      <c r="G57" s="6" t="s">
+        <v>155</v>
+      </c>
       <c r="H57" s="4" t="s">
-        <v>334</v>
+        <v>346</v>
       </c>
     </row>
     <row r="58" spans="1:8">
       <c r="A58" s="4" t="s">
-        <v>335</v>
+        <v>347</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>329</v>
+        <v>341</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>336</v>
+        <v>348</v>
       </c>
       <c r="D58" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E58" s="4" t="s">
-        <v>337</v>
+        <v>349</v>
       </c>
       <c r="F58" s="6"/>
-      <c r="G58" s="6"/>
+      <c r="G58" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H58" s="4" t="s">
-        <v>338</v>
+        <v>350</v>
       </c>
     </row>
     <row r="59" spans="1:8">
       <c r="A59" s="4" t="s">
-        <v>339</v>
+        <v>351</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>329</v>
+        <v>341</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>340</v>
+        <v>352</v>
       </c>
       <c r="D59" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E59" s="4" t="s">
-        <v>183</v>
+        <v>193</v>
       </c>
       <c r="F59" s="6"/>
-      <c r="G59" s="6"/>
+      <c r="G59" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H59" s="4" t="s">
-        <v>341</v>
+        <v>353</v>
       </c>
     </row>
     <row r="60" spans="1:8">
       <c r="A60" s="4" t="s">
-        <v>342</v>
+        <v>354</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>329</v>
+        <v>341</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>343</v>
+        <v>355</v>
       </c>
       <c r="D60" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E60" s="4" t="s">
-        <v>163</v>
+        <v>173</v>
       </c>
       <c r="F60" s="6"/>
-      <c r="G60" s="6"/>
+      <c r="G60" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H60" s="4" t="s">
-        <v>344</v>
+        <v>356</v>
       </c>
     </row>
     <row r="61" spans="1:8">
       <c r="A61" s="4" t="s">
-        <v>345</v>
+        <v>357</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>346</v>
+        <v>358</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>347</v>
+        <v>359</v>
       </c>
       <c r="D61" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E61" s="4" t="s">
-        <v>273</v>
+        <v>285</v>
       </c>
       <c r="F61" s="6"/>
-      <c r="G61" s="6"/>
+      <c r="G61" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H61" s="4" t="s">
-        <v>348</v>
+        <v>360</v>
       </c>
     </row>
     <row r="62" spans="1:8">
       <c r="A62" s="4" t="s">
-        <v>349</v>
+        <v>361</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>346</v>
+        <v>358</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>350</v>
+        <v>362</v>
       </c>
       <c r="D62" s="6" t="s">
-        <v>154</v>
+        <v>164</v>
       </c>
       <c r="E62" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="F62" s="6"/>
-      <c r="G62" s="6"/>
+        <v>147</v>
+      </c>
+      <c r="F62" s="6">
+        <v>19</v>
+      </c>
+      <c r="G62" s="6" t="s">
+        <v>155</v>
+      </c>
       <c r="H62" s="4" t="s">
-        <v>351</v>
+        <v>363</v>
       </c>
     </row>
     <row r="63" spans="1:8">
       <c r="A63" s="4" t="s">
-        <v>352</v>
+        <v>364</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>346</v>
+        <v>358</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>353</v>
+        <v>365</v>
       </c>
       <c r="D63" s="8" t="s">
-        <v>259</v>
+        <v>270</v>
       </c>
       <c r="E63" s="4" t="s">
-        <v>213</v>
+        <v>223</v>
       </c>
       <c r="F63" s="6"/>
-      <c r="G63" s="6"/>
+      <c r="G63" s="6" t="s">
+        <v>272</v>
+      </c>
       <c r="H63" s="4" t="s">
-        <v>354</v>
+        <v>366</v>
       </c>
     </row>
     <row r="64" spans="1:8">
       <c r="A64" s="4" t="s">
-        <v>355</v>
+        <v>367</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>346</v>
+        <v>358</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>356</v>
+        <v>368</v>
       </c>
       <c r="D64" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E64" s="4" t="s">
-        <v>357</v>
-      </c>
-      <c r="F64" s="6"/>
-      <c r="G64" s="6"/>
+        <v>369</v>
+      </c>
+      <c r="F64" s="6">
+        <v>15</v>
+      </c>
+      <c r="G64" s="6" t="s">
+        <v>155</v>
+      </c>
       <c r="H64" s="4" t="s">
-        <v>358</v>
+        <v>370</v>
       </c>
     </row>
     <row r="65" spans="1:8">
       <c r="A65" s="4" t="s">
-        <v>359</v>
+        <v>371</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>346</v>
+        <v>358</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>360</v>
+        <v>372</v>
       </c>
       <c r="D65" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E65" s="4" t="s">
-        <v>361</v>
+        <v>373</v>
       </c>
       <c r="F65" s="6"/>
-      <c r="G65" s="6"/>
+      <c r="G65" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H65" s="4" t="s">
-        <v>362</v>
+        <v>374</v>
       </c>
     </row>
     <row r="66" spans="1:8">
       <c r="A66" s="4" t="s">
-        <v>363</v>
+        <v>375</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>346</v>
+        <v>358</v>
       </c>
       <c r="C66" s="4" t="s">
-        <v>364</v>
+        <v>376</v>
       </c>
       <c r="D66" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E66" s="4" t="s">
-        <v>365</v>
-      </c>
-      <c r="F66" s="6"/>
-      <c r="G66" s="6"/>
+        <v>377</v>
+      </c>
+      <c r="F66" s="6">
+        <v>9</v>
+      </c>
+      <c r="G66" s="6" t="s">
+        <v>155</v>
+      </c>
       <c r="H66" s="4" t="s">
-        <v>366</v>
+        <v>378</v>
       </c>
     </row>
     <row r="67" spans="1:8">
       <c r="A67" s="4" t="s">
-        <v>367</v>
+        <v>379</v>
       </c>
       <c r="B67" s="4" t="s">
-        <v>346</v>
+        <v>358</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>368</v>
+        <v>380</v>
       </c>
       <c r="D67" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E67" s="4" t="s">
-        <v>369</v>
-      </c>
-      <c r="F67" s="6"/>
-      <c r="G67" s="6"/>
+        <v>381</v>
+      </c>
+      <c r="F67" s="6">
+        <v>5</v>
+      </c>
+      <c r="G67" s="6" t="s">
+        <v>228</v>
+      </c>
       <c r="H67" s="4" t="s">
-        <v>370</v>
+        <v>382</v>
       </c>
     </row>
     <row r="68" spans="1:8">
       <c r="A68" s="4" t="s">
-        <v>371</v>
+        <v>383</v>
       </c>
       <c r="B68" s="4" t="s">
-        <v>346</v>
+        <v>358</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>372</v>
+        <v>384</v>
       </c>
       <c r="D68" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E68" s="4" t="s">
-        <v>373</v>
-      </c>
-      <c r="F68" s="6"/>
-      <c r="G68" s="6"/>
+        <v>385</v>
+      </c>
+      <c r="F68" s="6">
+        <v>6</v>
+      </c>
+      <c r="G68" s="6" t="s">
+        <v>228</v>
+      </c>
       <c r="H68" s="4" t="s">
-        <v>374</v>
+        <v>386</v>
       </c>
     </row>
     <row r="69" spans="1:8">
       <c r="A69" s="4" t="s">
-        <v>375</v>
+        <v>387</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>346</v>
+        <v>358</v>
       </c>
       <c r="C69" s="4" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="D69" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E69" s="4" t="s">
-        <v>377</v>
+        <v>389</v>
       </c>
       <c r="F69" s="6"/>
-      <c r="G69" s="6"/>
+      <c r="G69" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H69" s="4" t="s">
-        <v>378</v>
+        <v>390</v>
       </c>
     </row>
     <row r="70" spans="1:8">
       <c r="A70" s="4" t="s">
-        <v>379</v>
+        <v>391</v>
       </c>
       <c r="B70" s="4" t="s">
-        <v>346</v>
+        <v>358</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>380</v>
+        <v>392</v>
       </c>
       <c r="D70" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E70" s="4" t="s">
-        <v>381</v>
+        <v>393</v>
       </c>
       <c r="F70" s="6"/>
-      <c r="G70" s="6"/>
+      <c r="G70" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H70" s="4" t="s">
-        <v>382</v>
+        <v>394</v>
       </c>
     </row>
     <row r="71" spans="1:8">
       <c r="A71" s="4" t="s">
-        <v>383</v>
+        <v>395</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>346</v>
+        <v>358</v>
       </c>
       <c r="C71" s="4" t="s">
-        <v>384</v>
+        <v>396</v>
       </c>
       <c r="D71" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E71" s="4" t="s">
-        <v>385</v>
+        <v>397</v>
       </c>
       <c r="F71" s="6"/>
-      <c r="G71" s="6"/>
+      <c r="G71" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H71" s="4" t="s">
-        <v>386</v>
+        <v>398</v>
       </c>
     </row>
     <row r="72" spans="1:8">
       <c r="A72" s="4" t="s">
-        <v>387</v>
+        <v>399</v>
       </c>
       <c r="B72" s="4" t="s">
-        <v>346</v>
+        <v>358</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>388</v>
+        <v>400</v>
       </c>
       <c r="D72" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E72" s="4" t="s">
-        <v>389</v>
+        <v>401</v>
       </c>
       <c r="F72" s="6"/>
-      <c r="G72" s="6"/>
+      <c r="G72" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H72" s="4" t="s">
-        <v>313</v>
+        <v>325</v>
       </c>
     </row>
     <row r="73" spans="1:8">
       <c r="A73" s="4" t="s">
-        <v>390</v>
+        <v>402</v>
       </c>
       <c r="B73" s="4" t="s">
-        <v>346</v>
+        <v>358</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>391</v>
+        <v>403</v>
       </c>
       <c r="D73" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E73" s="4" t="s">
-        <v>392</v>
+        <v>404</v>
       </c>
       <c r="F73" s="6"/>
-      <c r="G73" s="6"/>
+      <c r="G73" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H73" s="4"/>
     </row>
     <row r="74" spans="1:8">
       <c r="A74" s="4" t="s">
-        <v>393</v>
+        <v>405</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>346</v>
+        <v>358</v>
       </c>
       <c r="C74" s="4" t="s">
-        <v>394</v>
+        <v>406</v>
       </c>
       <c r="D74" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E74" s="4" t="s">
-        <v>395</v>
+        <v>407</v>
       </c>
       <c r="F74" s="6"/>
-      <c r="G74" s="6"/>
+      <c r="G74" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H74" s="4" t="s">
-        <v>396</v>
+        <v>408</v>
       </c>
     </row>
     <row r="75" spans="1:8">
       <c r="A75" s="4" t="s">
-        <v>397</v>
+        <v>409</v>
       </c>
       <c r="B75" s="4" t="s">
-        <v>398</v>
+        <v>410</v>
       </c>
       <c r="C75" s="4" t="s">
-        <v>399</v>
+        <v>411</v>
       </c>
       <c r="D75" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E75" s="4" t="s">
-        <v>400</v>
-      </c>
-      <c r="F75" s="6"/>
-      <c r="G75" s="6"/>
+        <v>412</v>
+      </c>
+      <c r="F75" s="6">
+        <v>1</v>
+      </c>
+      <c r="G75" s="6" t="s">
+        <v>228</v>
+      </c>
       <c r="H75" s="4" t="s">
-        <v>401</v>
+        <v>413</v>
       </c>
     </row>
     <row r="76" spans="1:8">
       <c r="A76" s="4" t="s">
-        <v>402</v>
+        <v>414</v>
       </c>
       <c r="B76" s="4" t="s">
-        <v>403</v>
+        <v>415</v>
       </c>
       <c r="C76" s="4" t="s">
-        <v>404</v>
+        <v>416</v>
       </c>
       <c r="D76" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E76" s="4" t="s">
-        <v>405</v>
+        <v>417</v>
       </c>
       <c r="F76" s="6"/>
-      <c r="G76" s="6"/>
+      <c r="G76" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H76" s="4"/>
     </row>
     <row r="77" spans="1:8">
       <c r="A77" s="4" t="s">
-        <v>406</v>
+        <v>418</v>
       </c>
       <c r="B77" s="4" t="s">
-        <v>403</v>
+        <v>415</v>
       </c>
       <c r="C77" s="4" t="s">
-        <v>407</v>
+        <v>419</v>
       </c>
       <c r="D77" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E77" s="4" t="s">
-        <v>408</v>
-      </c>
-      <c r="F77" s="6"/>
-      <c r="G77" s="6"/>
+        <v>420</v>
+      </c>
+      <c r="F77" s="6">
+        <v>7</v>
+      </c>
+      <c r="G77" s="6" t="s">
+        <v>228</v>
+      </c>
       <c r="H77" s="4" t="s">
-        <v>409</v>
+        <v>421</v>
       </c>
     </row>
     <row r="78" spans="1:8">
       <c r="A78" s="4" t="s">
-        <v>410</v>
+        <v>422</v>
       </c>
       <c r="B78" s="4" t="s">
-        <v>403</v>
+        <v>415</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>411</v>
+        <v>423</v>
       </c>
       <c r="D78" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E78" s="4" t="s">
-        <v>412</v>
+        <v>424</v>
       </c>
       <c r="F78" s="6"/>
-      <c r="G78" s="6"/>
+      <c r="G78" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="H78" s="4" t="s">
-        <v>413</v>
+        <v>425</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: binary V1/V2 split in workbook (drop fuzzy v1.x)
Per feedback: every item is V1 or V2, no in-between. The tab IS the version —
'V1 - Next launch' and 'V2 - Future'. Removed the per-row version column and all
'v1.x'/'soon' wording; the 4 ex-'soon' items become V2. User columns still read
live + preserved (sheet-name-agnostic reader).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/finwise-launch-and-parked.xlsx
+++ b/docs/finwise-launch-and-parked.xlsx
@@ -7,24 +7,24 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Launch (v1)" sheetId="1" r:id="rId1"/>
-    <sheet name="Future backlog" sheetId="2" r:id="rId2"/>
+    <sheet name="V1 — Next launch" sheetId="1" r:id="rId1"/>
+    <sheet name="V2 — Future" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Future backlog'!$A$4:$H$47</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Launch (v1)'!$A$4:$L$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'V1 — Next launch'!$A$4:$L$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'V2 — Future'!$A$4:$G$47</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="809" uniqueCount="396">
-  <si>
-    <t>Launch (v1)</t>
-  </si>
-  <si>
-    <t>Everything targeted for the NEXT launch (v1): the must-do steps to ship, PLUS the v1 work lifted up from the backlog. Type: 'Blocker' = can't ship without it · 'v1 feature' = wanted in the launch but not blocking the submission · 'Important'/'Decision'/'Recommended' as labelled. Stage = where it is (Plan→Design→Build→Test→Refine→Ready, or Done). The top block (L-#) is the ship process in critical-path order; below it are the v1 features. Yellow columns are yours to fill (J Rank / J Notes / Decision); 'Your rank' is my suggested order. Heads-up: the must-ship-to-submit set is the Blockers near the top — the v1 features can't all make a launch that's days away.</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="765" uniqueCount="393">
+  <si>
+    <t>V1 — Next launch</t>
+  </si>
+  <si>
+    <t>EVERYTHING ON THIS TAB IS V1 (the next launch). It has the must-do steps to ship PLUS the v1 work lifted up from the backlog. Type: 'Blocker' = can't ship without it · 'v1 feature' = wanted in the launch but not blocking the submission · 'Important'/'Decision'/'Recommended' as labelled. Stage = where it is (Plan→Design→Build→Test→Refine→Ready, or Done). The top block (L-#) is the ship process in critical-path order; below it are the v1 features. Yellow columns are yours (J Rank / J Notes / Decision); 'Your rank' is my suggested order. To push something to a future release, tell me and I'll move it to the V2 tab. Heads-up: the must-ship set is the Blockers near the top — the 24 v1 features can't all make a launch that's days away.</t>
   </si>
   <si>
     <t>ID</t>
@@ -783,10 +783,10 @@
     <t>Easier to read for some users; lower priority.</t>
   </si>
   <si>
-    <t>Future backlog</t>
-  </si>
-  <si>
-    <t>Everything NOT in the next launch — future work, grouped by area. Version: 'v1.x (soon)' = a soon-after-launch point release · 'v2 (future)' = a later bigger release. Stage shows how far along each is; 'What's left' spells out what's unfinished for the part-done ones. Yellow columns are yours (Version / Your notes). Note: I lifted every v1 item up to the Launch tab, and removed the crash-reporting row here because it's the same work as a launch item (L-12).</t>
+    <t>V2 — Future</t>
+  </si>
+  <si>
+    <t>EVERYTHING ON THIS TAB IS V2 (a future release, after the next launch) — grouped by area. There is no in-between: if it's not here, it's in V1. Stage shows how far along each is; 'What's left' spells out what's unfinished for the part-done ones. The yellow 'Your notes' column is yours. To pull any of these INTO the next launch, tell me and I'll move it to the V1 tab. (I removed the crash-reporting row — it's the same work as launch item L-12.)</t>
   </si>
   <si>
     <t>Category</t>
@@ -795,9 +795,6 @@
     <t>What's left</t>
   </si>
   <si>
-    <t>Version (v1.x soon / v2 future)</t>
-  </si>
-  <si>
     <t>Your notes</t>
   </si>
   <si>
@@ -810,9 +807,6 @@
     <t>Connect the app to your bank and brokerage so balances and transactions pull in automatically.</t>
   </si>
   <si>
-    <t>v2 (future)</t>
-  </si>
-  <si>
     <t>Biggest convenience and stickiness win, but a large build needing a secure server.</t>
   </si>
   <si>
@@ -1054,9 +1048,6 @@
   </si>
   <si>
     <t>The goals tab and funding logic exist; the full visual screen isn't finished.</t>
-  </si>
-  <si>
-    <t>v1.x (soon)</t>
   </si>
   <si>
     <t>Helps people set and track goals; a stickiness feature.</t>
@@ -3699,7 +3690,7 @@
   <sheetPr>
     <tabColor rgb="FF1F4E5F"/>
   </sheetPr>
-  <dimension ref="A1:H47"/>
+  <dimension ref="A1:G47"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="6.7109375" customWidth="1"/>
@@ -3707,12 +3698,11 @@
     <col min="3" max="3" width="52.7109375" customWidth="1"/>
     <col min="4" max="4" width="8.7109375" customWidth="1"/>
     <col min="5" max="5" width="34.7109375" customWidth="1"/>
-    <col min="6" max="6" width="20.7109375" customWidth="1"/>
-    <col min="7" max="7" width="18.7109375" customWidth="1"/>
-    <col min="8" max="8" width="50.7109375" customWidth="1"/>
+    <col min="6" max="6" width="18.7109375" customWidth="1"/>
+    <col min="7" max="7" width="52.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
         <v>254</v>
       </c>
@@ -3722,9 +3712,8 @@
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-    </row>
-    <row r="2" spans="1:8" ht="28" customHeight="1">
+    </row>
+    <row r="2" spans="1:7" ht="28" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>255</v>
       </c>
@@ -3734,9 +3723,8 @@
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-    </row>
-    <row r="3" spans="1:8">
+    </row>
+    <row r="3" spans="1:7">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -3744,9 +3732,8 @@
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-    </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1">
+    </row>
+    <row r="4" spans="1:7" ht="30" customHeight="1">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -3768,967 +3755,835 @@
       <c r="G4" s="3" t="s">
         <v>259</v>
       </c>
-      <c r="H4" s="3" t="s">
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" s="4" t="s">
         <v>260</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8">
-      <c r="A5" s="4" t="s">
-        <v>261</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>15</v>
       </c>
       <c r="C5" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="4"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="4" t="s">
         <v>262</v>
       </c>
-      <c r="D5" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E5" s="4"/>
-      <c r="F5" s="6" t="s">
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" s="4" t="s">
         <v>263</v>
-      </c>
-      <c r="G5" s="6"/>
-      <c r="H5" s="4" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8">
-      <c r="A6" s="4" t="s">
-        <v>265</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>15</v>
       </c>
       <c r="C6" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" s="4"/>
+      <c r="F6" s="6"/>
+      <c r="G6" s="4" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" s="4" t="s">
         <v>266</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E6" s="4"/>
-      <c r="F6" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="G6" s="6"/>
-      <c r="H6" s="4" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8">
-      <c r="A7" s="4" t="s">
-        <v>268</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>15</v>
       </c>
       <c r="C7" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" s="4"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="4" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" s="4" t="s">
         <v>269</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E7" s="4"/>
-      <c r="F7" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="G7" s="6"/>
-      <c r="H7" s="4" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8">
-      <c r="A8" s="4" t="s">
-        <v>271</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>178</v>
       </c>
       <c r="C8" s="4" t="s">
+        <v>270</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E8" s="4"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="4" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" s="4" t="s">
         <v>272</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E8" s="4"/>
-      <c r="F8" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="G8" s="6"/>
-      <c r="H8" s="4" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8">
-      <c r="A9" s="4" t="s">
-        <v>274</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>189</v>
       </c>
       <c r="C9" s="4" t="s">
+        <v>273</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E9" s="4"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="4" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" s="4" t="s">
         <v>275</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E9" s="4"/>
-      <c r="F9" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="G9" s="6"/>
-      <c r="H9" s="4" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8">
-      <c r="A10" s="4" t="s">
-        <v>277</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>189</v>
       </c>
       <c r="C10" s="4" t="s">
+        <v>276</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" s="4"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="4" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" s="4" t="s">
         <v>278</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E10" s="4"/>
-      <c r="F10" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="G10" s="6"/>
-      <c r="H10" s="4" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8">
-      <c r="A11" s="4" t="s">
-        <v>280</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>189</v>
       </c>
       <c r="C11" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E11" s="4"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="4" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" s="4" t="s">
         <v>281</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E11" s="4"/>
-      <c r="F11" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="G11" s="6"/>
-      <c r="H11" s="4" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8">
-      <c r="A12" s="4" t="s">
-        <v>283</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>189</v>
       </c>
       <c r="C12" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" s="4"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="4" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" s="4" t="s">
         <v>284</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E12" s="4"/>
-      <c r="F12" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="G12" s="6"/>
-      <c r="H12" s="4" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8">
-      <c r="A13" s="4" t="s">
-        <v>286</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>45</v>
       </c>
       <c r="C13" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E13" s="4"/>
+      <c r="F13" s="6"/>
+      <c r="G13" s="4" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" s="4" t="s">
         <v>287</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E13" s="4"/>
-      <c r="F13" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="G13" s="6"/>
-      <c r="H13" s="4" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8">
-      <c r="A14" s="4" t="s">
-        <v>289</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>45</v>
       </c>
       <c r="C14" s="4" t="s">
+        <v>288</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E14" s="4"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="4" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15" s="4" t="s">
         <v>290</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E14" s="4"/>
-      <c r="F14" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="G14" s="6"/>
-      <c r="H14" s="4" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8">
-      <c r="A15" s="4" t="s">
-        <v>292</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>45</v>
       </c>
       <c r="C15" s="4" t="s">
+        <v>291</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E15" s="4"/>
+      <c r="F15" s="6"/>
+      <c r="G15" s="4" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16" s="4" t="s">
         <v>293</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E15" s="4"/>
-      <c r="F15" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="G15" s="6"/>
-      <c r="H15" s="4" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8">
-      <c r="A16" s="4" t="s">
-        <v>295</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>45</v>
       </c>
       <c r="C16" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E16" s="4"/>
+      <c r="F16" s="6"/>
+      <c r="G16" s="4" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17" s="4" t="s">
         <v>296</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E16" s="4"/>
-      <c r="F16" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="G16" s="6"/>
-      <c r="H16" s="4" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8">
-      <c r="A17" s="4" t="s">
-        <v>298</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>155</v>
       </c>
       <c r="C17" s="4" t="s">
+        <v>297</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E17" s="4"/>
+      <c r="F17" s="6"/>
+      <c r="G17" s="4" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18" s="4" t="s">
         <v>299</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E17" s="4"/>
-      <c r="F17" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="G17" s="6"/>
-      <c r="H17" s="4" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8">
-      <c r="A18" s="4" t="s">
-        <v>301</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>155</v>
       </c>
       <c r="C18" s="4" t="s">
+        <v>300</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E18" s="4"/>
+      <c r="F18" s="6"/>
+      <c r="G18" s="4" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19" s="4" t="s">
         <v>302</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E18" s="4"/>
-      <c r="F18" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="G18" s="6"/>
-      <c r="H18" s="4" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8">
-      <c r="A19" s="4" t="s">
-        <v>304</v>
       </c>
       <c r="B19" s="4" t="s">
         <v>155</v>
       </c>
       <c r="C19" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E19" s="4"/>
+      <c r="F19" s="6"/>
+      <c r="G19" s="4" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20" s="4" t="s">
         <v>305</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E19" s="4"/>
-      <c r="F19" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="G19" s="6"/>
-      <c r="H19" s="4" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8">
-      <c r="A20" s="4" t="s">
-        <v>307</v>
       </c>
       <c r="B20" s="4" t="s">
         <v>155</v>
       </c>
       <c r="C20" s="4" t="s">
+        <v>306</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E20" s="4"/>
+      <c r="F20" s="6"/>
+      <c r="G20" s="4" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" s="4" t="s">
         <v>308</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E20" s="4"/>
-      <c r="F20" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="G20" s="6"/>
-      <c r="H20" s="4" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8">
-      <c r="A21" s="4" t="s">
-        <v>310</v>
       </c>
       <c r="B21" s="4" t="s">
         <v>221</v>
       </c>
       <c r="C21" s="4" t="s">
+        <v>309</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E21" s="4"/>
+      <c r="F21" s="6"/>
+      <c r="G21" s="4" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" s="4" t="s">
         <v>311</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E21" s="4"/>
-      <c r="F21" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="G21" s="6"/>
-      <c r="H21" s="4" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8">
-      <c r="A22" s="4" t="s">
-        <v>313</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>221</v>
       </c>
       <c r="C22" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E22" s="4"/>
+      <c r="F22" s="6"/>
+      <c r="G22" s="4" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23" s="4" t="s">
         <v>314</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E22" s="4"/>
-      <c r="F22" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="G22" s="6"/>
-      <c r="H22" s="4" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8">
-      <c r="A23" s="4" t="s">
-        <v>316</v>
       </c>
       <c r="B23" s="4" t="s">
         <v>221</v>
       </c>
       <c r="C23" s="4" t="s">
+        <v>315</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E23" s="4"/>
+      <c r="F23" s="6"/>
+      <c r="G23" s="4" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7">
+      <c r="A24" s="4" t="s">
         <v>317</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E23" s="4"/>
-      <c r="F23" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="G23" s="6"/>
-      <c r="H23" s="4" t="s">
-        <v>318</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8">
-      <c r="A24" s="4" t="s">
-        <v>319</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>221</v>
       </c>
       <c r="C24" s="4" t="s">
+        <v>318</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E24" s="4"/>
+      <c r="F24" s="6"/>
+      <c r="G24" s="4" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
+      <c r="A25" s="4" t="s">
         <v>320</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E24" s="4"/>
-      <c r="F24" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="G24" s="6"/>
-      <c r="H24" s="4" t="s">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8">
-      <c r="A25" s="4" t="s">
-        <v>322</v>
       </c>
       <c r="B25" s="4" t="s">
         <v>221</v>
       </c>
       <c r="C25" s="4" t="s">
+        <v>321</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E25" s="4"/>
+      <c r="F25" s="6"/>
+      <c r="G25" s="4" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7">
+      <c r="A26" s="4" t="s">
         <v>323</v>
-      </c>
-      <c r="D25" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E25" s="4"/>
-      <c r="F25" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="G25" s="6"/>
-      <c r="H25" s="4" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
-      <c r="A26" s="4" t="s">
-        <v>325</v>
       </c>
       <c r="B26" s="4" t="s">
         <v>221</v>
       </c>
       <c r="C26" s="4" t="s">
+        <v>324</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E26" s="4"/>
+      <c r="F26" s="6"/>
+      <c r="G26" s="4" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7">
+      <c r="A27" s="4" t="s">
         <v>326</v>
-      </c>
-      <c r="D26" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E26" s="4"/>
-      <c r="F26" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="G26" s="6"/>
-      <c r="H26" s="4" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8">
-      <c r="A27" s="4" t="s">
-        <v>328</v>
       </c>
       <c r="B27" s="4" t="s">
         <v>221</v>
       </c>
       <c r="C27" s="4" t="s">
+        <v>327</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E27" s="4"/>
+      <c r="F27" s="6"/>
+      <c r="G27" s="4" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7">
+      <c r="A28" s="4" t="s">
         <v>329</v>
-      </c>
-      <c r="D27" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E27" s="4"/>
-      <c r="F27" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="G27" s="6"/>
-      <c r="H27" s="4" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8">
-      <c r="A28" s="4" t="s">
-        <v>331</v>
       </c>
       <c r="B28" s="4" t="s">
         <v>221</v>
       </c>
       <c r="C28" s="4" t="s">
+        <v>330</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E28" s="4"/>
+      <c r="F28" s="6"/>
+      <c r="G28" s="4" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="A29" s="4" t="s">
         <v>332</v>
-      </c>
-      <c r="D28" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E28" s="4"/>
-      <c r="F28" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="G28" s="6"/>
-      <c r="H28" s="4" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8">
-      <c r="A29" s="4" t="s">
-        <v>334</v>
       </c>
       <c r="B29" s="4" t="s">
         <v>221</v>
       </c>
       <c r="C29" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E29" s="4"/>
+      <c r="F29" s="6"/>
+      <c r="G29" s="4" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7">
+      <c r="A30" s="4" t="s">
         <v>335</v>
       </c>
-      <c r="D29" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E29" s="4"/>
-      <c r="F29" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="G29" s="6"/>
-      <c r="H29" s="4" t="s">
+      <c r="B30" s="4" t="s">
         <v>336</v>
       </c>
-    </row>
-    <row r="30" spans="1:8">
-      <c r="A30" s="4" t="s">
+      <c r="C30" s="4" t="s">
         <v>337</v>
       </c>
-      <c r="B30" s="4" t="s">
+      <c r="D30" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E30" s="4" t="s">
         <v>338</v>
       </c>
-      <c r="C30" s="4" t="s">
+      <c r="F30" s="6"/>
+      <c r="G30" s="4" t="s">
         <v>339</v>
       </c>
-      <c r="D30" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E30" s="4" t="s">
+    </row>
+    <row r="31" spans="1:7">
+      <c r="A31" s="4" t="s">
         <v>340</v>
       </c>
-      <c r="F30" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="G30" s="6"/>
-      <c r="H30" s="4" t="s">
+      <c r="B31" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="C31" s="4" t="s">
         <v>341</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8">
-      <c r="A31" s="4" t="s">
-        <v>342</v>
-      </c>
-      <c r="B31" s="4" t="s">
-        <v>338</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>343</v>
       </c>
       <c r="D31" s="10" t="s">
         <v>76</v>
       </c>
       <c r="E31" s="4" t="s">
+        <v>342</v>
+      </c>
+      <c r="F31" s="6"/>
+      <c r="G31" s="4" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7">
+      <c r="A32" s="4" t="s">
         <v>344</v>
       </c>
-      <c r="F31" s="6" t="s">
+      <c r="B32" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="C32" s="4" t="s">
         <v>345</v>
       </c>
-      <c r="G31" s="6"/>
-      <c r="H31" s="4" t="s">
+      <c r="D32" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E32" s="4"/>
+      <c r="F32" s="6"/>
+      <c r="G32" s="4" t="s">
         <v>346</v>
       </c>
     </row>
-    <row r="32" spans="1:8">
-      <c r="A32" s="4" t="s">
+    <row r="33" spans="1:7">
+      <c r="A33" s="4" t="s">
         <v>347</v>
       </c>
-      <c r="B32" s="4" t="s">
-        <v>338</v>
-      </c>
-      <c r="C32" s="4" t="s">
+      <c r="B33" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="C33" s="4" t="s">
         <v>348</v>
       </c>
-      <c r="D32" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E32" s="4"/>
-      <c r="F32" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="G32" s="6"/>
-      <c r="H32" s="4" t="s">
+      <c r="D33" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E33" s="4"/>
+      <c r="F33" s="6"/>
+      <c r="G33" s="4" t="s">
         <v>349</v>
       </c>
     </row>
-    <row r="33" spans="1:8">
-      <c r="A33" s="4" t="s">
+    <row r="34" spans="1:7">
+      <c r="A34" s="4" t="s">
         <v>350</v>
       </c>
-      <c r="B33" s="4" t="s">
-        <v>338</v>
-      </c>
-      <c r="C33" s="4" t="s">
+      <c r="B34" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="C34" s="4" t="s">
         <v>351</v>
       </c>
-      <c r="D33" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E33" s="4"/>
-      <c r="F33" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="G33" s="6"/>
-      <c r="H33" s="4" t="s">
+      <c r="D34" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E34" s="4"/>
+      <c r="F34" s="6"/>
+      <c r="G34" s="4" t="s">
         <v>352</v>
       </c>
     </row>
-    <row r="34" spans="1:8">
-      <c r="A34" s="4" t="s">
+    <row r="35" spans="1:7">
+      <c r="A35" s="4" t="s">
         <v>353</v>
-      </c>
-      <c r="B34" s="4" t="s">
-        <v>338</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>354</v>
-      </c>
-      <c r="D34" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E34" s="4"/>
-      <c r="F34" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="G34" s="6"/>
-      <c r="H34" s="4" t="s">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8">
-      <c r="A35" s="4" t="s">
-        <v>356</v>
       </c>
       <c r="B35" s="4" t="s">
         <v>159</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="D35" s="5" t="s">
         <v>19</v>
       </c>
       <c r="E35" s="4"/>
-      <c r="F35" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="G35" s="6"/>
-      <c r="H35" s="4" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8">
+      <c r="F35" s="6"/>
+      <c r="G35" s="4" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7">
       <c r="A36" s="4" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="B36" s="4" t="s">
         <v>159</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="D36" s="10" t="s">
         <v>76</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>361</v>
-      </c>
-      <c r="F36" s="6" t="s">
-        <v>345</v>
-      </c>
-      <c r="G36" s="6"/>
-      <c r="H36" s="4" t="s">
-        <v>362</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8">
+        <v>358</v>
+      </c>
+      <c r="F36" s="6"/>
+      <c r="G36" s="4" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7">
       <c r="A37" s="4" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="B37" s="4" t="s">
         <v>159</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="D37" s="5" t="s">
         <v>19</v>
       </c>
       <c r="E37" s="4"/>
-      <c r="F37" s="6" t="s">
-        <v>345</v>
-      </c>
-      <c r="G37" s="6"/>
-      <c r="H37" s="4" t="s">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8">
+      <c r="F37" s="6"/>
+      <c r="G37" s="4" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7">
       <c r="A38" s="4" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="B38" s="4" t="s">
         <v>159</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="D38" s="5" t="s">
         <v>19</v>
       </c>
       <c r="E38" s="4"/>
-      <c r="F38" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="G38" s="6"/>
-      <c r="H38" s="4" t="s">
-        <v>368</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8">
+      <c r="F38" s="6"/>
+      <c r="G38" s="4" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7">
       <c r="A39" s="4" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="B39" s="4" t="s">
         <v>159</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="D39" s="5" t="s">
         <v>19</v>
       </c>
       <c r="E39" s="4"/>
-      <c r="F39" s="6" t="s">
-        <v>345</v>
-      </c>
-      <c r="G39" s="6"/>
-      <c r="H39" s="4" t="s">
-        <v>371</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8">
+      <c r="F39" s="6"/>
+      <c r="G39" s="4" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7">
       <c r="A40" s="4" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="B40" s="4" t="s">
         <v>159</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="D40" s="5" t="s">
         <v>19</v>
       </c>
       <c r="E40" s="4"/>
-      <c r="F40" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="G40" s="6"/>
-      <c r="H40" s="4" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8">
+      <c r="F40" s="6"/>
+      <c r="G40" s="4" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7">
       <c r="A41" s="4" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="B41" s="4" t="s">
         <v>159</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="D41" s="5" t="s">
         <v>19</v>
       </c>
       <c r="E41" s="4"/>
-      <c r="F41" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="G41" s="6"/>
-      <c r="H41" s="4" t="s">
-        <v>377</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8">
+      <c r="F41" s="6"/>
+      <c r="G41" s="4" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7">
       <c r="A42" s="4" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="B42" s="4" t="s">
         <v>159</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="D42" s="5" t="s">
         <v>19</v>
       </c>
       <c r="E42" s="4"/>
-      <c r="F42" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="G42" s="6"/>
-      <c r="H42" s="4" t="s">
-        <v>380</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8">
+      <c r="F42" s="6"/>
+      <c r="G42" s="4" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7">
       <c r="A43" s="4" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="B43" s="4" t="s">
         <v>159</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="D43" s="5" t="s">
         <v>19</v>
       </c>
       <c r="E43" s="4"/>
-      <c r="F43" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="G43" s="6"/>
-      <c r="H43" s="4" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8">
+      <c r="F43" s="6"/>
+      <c r="G43" s="4" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7">
       <c r="A44" s="4" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="B44" s="4" t="s">
         <v>159</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="D44" s="5" t="s">
         <v>19</v>
       </c>
       <c r="E44" s="4"/>
-      <c r="F44" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="G44" s="6"/>
-      <c r="H44" s="4" t="s">
-        <v>386</v>
-      </c>
-    </row>
-    <row r="45" spans="1:8">
+      <c r="F44" s="6"/>
+      <c r="G44" s="4" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7">
       <c r="A45" s="4" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="B45" s="4" t="s">
         <v>159</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="D45" s="5" t="s">
         <v>19</v>
       </c>
       <c r="E45" s="4"/>
-      <c r="F45" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="G45" s="6"/>
-      <c r="H45" s="4" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="46" spans="1:8">
+      <c r="F45" s="6"/>
+      <c r="G45" s="4" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7">
       <c r="A46" s="4" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="B46" s="4" t="s">
         <v>166</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="D46" s="5" t="s">
         <v>19</v>
       </c>
       <c r="E46" s="4"/>
-      <c r="F46" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="G46" s="6"/>
-      <c r="H46" s="4" t="s">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="47" spans="1:8">
+      <c r="F46" s="6"/>
+      <c r="G46" s="4" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7">
       <c r="A47" s="4" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="B47" s="4" t="s">
         <v>166</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="D47" s="5" t="s">
         <v>19</v>
       </c>
       <c r="E47" s="4"/>
-      <c r="F47" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="G47" s="6"/>
-      <c r="H47" s="4" t="s">
-        <v>395</v>
+      <c r="F47" s="6"/>
+      <c r="G47" s="4" t="s">
+        <v>392</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:H47"/>
+  <autoFilter ref="A4:G47"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H3"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: three-bucket triage — V1 / Fast follow-up / V2
Per feedback, re-triaged all 100 items into three tabs:
- V1 - Next launch (30): the L-# ship process + only the true must-ship backlog
  (final app name [legal], two safety items, one already-built feature).
- Fast follow-up (13): my recommendation for the first quick post-launch update,
  in priority order (core-calc tests, spend reconciliation, network timeouts,
  analytics, receipt-scan tuning, CSV validation, goals UI, a11y x2, undo,
  loading states, runway, data export).
- V2 - Future (56): everything else (bank linking, copilot, couples, etc.).
No cross-tab dupes; P-59 stays dropped; user columns preserved.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/finwise-launch-and-parked.xlsx
+++ b/docs/finwise-launch-and-parked.xlsx
@@ -8,23 +8,25 @@
   </bookViews>
   <sheets>
     <sheet name="V1 — Next launch" sheetId="1" r:id="rId1"/>
-    <sheet name="V2 — Future" sheetId="2" r:id="rId2"/>
+    <sheet name="Fast follow-up" sheetId="2" r:id="rId2"/>
+    <sheet name="V2 — Future" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'V1 — Next launch'!$A$4:$L$60</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'V2 — Future'!$A$4:$G$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fast follow-up'!$A$4:$G$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'V1 — Next launch'!$A$4:$L$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'V2 — Future'!$A$4:$G$60</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="765" uniqueCount="393">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="676" uniqueCount="394">
   <si>
     <t>V1 — Next launch</t>
   </si>
   <si>
-    <t>EVERYTHING ON THIS TAB IS V1 (the next launch). It has the must-do steps to ship PLUS the v1 work lifted up from the backlog. Type: 'Blocker' = can't ship without it · 'v1 feature' = wanted in the launch but not blocking the submission · 'Important'/'Decision'/'Recommended' as labelled. Stage = where it is (Plan→Design→Build→Test→Refine→Ready, or Done). The top block (L-#) is the ship process in critical-path order; below it are the v1 features. Yellow columns are yours (J Rank / J Notes / Decision); 'Your rank' is my suggested order. To push something to a future release, tell me and I'll move it to the V2 tab. Heads-up: the must-ship set is the Blockers near the top — the 24 v1 features can't all make a launch that's days away.</t>
+    <t>EVERYTHING ON THIS TAB IS V1 — the genuine must-ship list for the next launch, nothing optional. It's the ship process (L-#, in critical-path order) plus the only backlog items that truly can't wait: the final app name (legal), two safety items, and one feature that's already built. Type: 'Blocker' = can't ship without it · 'Important' = strongly recommended before submit · 'Decision'/'Recommended' as labelled. Stage = where it is (Plan→Design→Build→Test→Refine→Ready, or Done). Yellow columns are yours (J Rank / J Notes / Decision); 'Your rank' is my suggested order. Things I'd do right after launch are on the 'Fast follow-up' tab; everything else is on 'V2 — Future'.</t>
   </si>
   <si>
     <t>ID</t>
@@ -477,79 +479,220 @@
     <t>Scan the app's building blocks for known security holes and fix the risky ones.</t>
   </si>
   <si>
-    <t>Before submit</t>
+    <t>Before submit — safety</t>
   </si>
   <si>
     <t>A high-priority safety check before launch.</t>
   </si>
   <si>
+    <t>P-63</t>
+  </si>
+  <si>
+    <t>Quality</t>
+  </si>
+  <si>
+    <t>Review that every data fetch handles errors gracefully, not just the happy path.</t>
+  </si>
+  <si>
+    <t>Prevents crashes and blank screens; high priority.</t>
+  </si>
+  <si>
+    <t>P-33</t>
+  </si>
+  <si>
+    <t>UI/UX</t>
+  </si>
+  <si>
+    <t>Add a tap to hide or blur your balances for privacy.</t>
+  </si>
+  <si>
+    <t>v1 feature</t>
+  </si>
+  <si>
+    <t>Done — verify</t>
+  </si>
+  <si>
+    <t>Lets you check the app in public without showing your money.</t>
+  </si>
+  <si>
+    <t>Fast follow-up</t>
+  </si>
+  <si>
+    <t>MY RECOMMENDATION for the first quick update right after launch — high-value, lower-risk improvements that don't block the launch but I'd ship soon after. Listed in priority order (top = first). These were pulled out of the backlog so they don't get lost behind the bigger V2 work. Want any of these IN the launch instead? Tell me and I'll move it to V1. Want one pushed further out? It goes to V2.</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>What's left</t>
+  </si>
+  <si>
+    <t>Your notes</t>
+  </si>
+  <si>
+    <t>Why it matters</t>
+  </si>
+  <si>
+    <t>P-62</t>
+  </si>
+  <si>
+    <t>Add tests for the core retirement and investment math.</t>
+  </si>
+  <si>
+    <t>Protects accuracy of the most important calculations; high priority.</t>
+  </si>
+  <si>
+    <t>P-38</t>
+  </si>
+  <si>
+    <t>Make total spending and the category breakdown always add up to the same number.</t>
+  </si>
+  <si>
+    <t>Prevents confusing double-counting between summaries and budget.</t>
+  </si>
+  <si>
+    <t>P-64</t>
+  </si>
+  <si>
+    <t>Add timeouts and retries so the app never hangs waiting on data.</t>
+  </si>
+  <si>
+    <t>Stops endless loading spinners; medium priority.</t>
+  </si>
+  <si>
+    <t>P-73</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>Add usage tracking to see how many people finish setup and keep coming back.</t>
+  </si>
+  <si>
+    <t>Needed to measure success and the top launch metric.</t>
+  </si>
+  <si>
+    <t>P-4</t>
+  </si>
+  <si>
+    <t>Turn on snap-a-photo receipt scanning and improve how it reads the totals.</t>
+  </si>
+  <si>
+    <t>Nearly ready; needs a real device build to switch on and test.</t>
+  </si>
+  <si>
+    <t>P-5</t>
+  </si>
+  <si>
+    <t>Catch bad rows when you import a spreadsheet so imports don't break things.</t>
+  </si>
+  <si>
+    <t>Protects against messy files corrupting your data.</t>
+  </si>
+  <si>
+    <t>P-53</t>
+  </si>
+  <si>
+    <t>Growth</t>
+  </si>
+  <si>
+    <t>Finish the full savings-goals screen with progress, priority, and projections.</t>
+  </si>
+  <si>
+    <t>The goals tab and funding logic exist; the full visual screen isn't finished.</t>
+  </si>
+  <si>
+    <t>Helps people set and track goals; a stickiness feature.</t>
+  </si>
+  <si>
+    <t>P-28</t>
+  </si>
+  <si>
+    <t>Accessibility</t>
+  </si>
+  <si>
+    <t>Make every screen work with the screen reader for blind and low-vision users.</t>
+  </si>
+  <si>
+    <t>The single biggest accessibility gap (for users with disabilities).</t>
+  </si>
+  <si>
     <t>P-29</t>
   </si>
   <si>
-    <t>Accessibility</t>
-  </si>
-  <si>
     <t>Make buttons big enough to tap reliably for everyone.</t>
   </si>
   <si>
     <t>An accessibility basic (for users with disabilities); high priority.</t>
   </si>
   <si>
-    <t>P-63</t>
-  </si>
-  <si>
-    <t>Quality</t>
-  </si>
-  <si>
-    <t>Review that every data fetch handles errors gracefully, not just the happy path.</t>
-  </si>
-  <si>
-    <t>Prevents crashes and blank screens; high priority.</t>
-  </si>
-  <si>
-    <t>P-64</t>
-  </si>
-  <si>
-    <t>Add timeouts and retries so the app never hangs waiting on data.</t>
-  </si>
-  <si>
-    <t>Stops endless loading spinners; medium priority.</t>
-  </si>
-  <si>
-    <t>P-73</t>
-  </si>
-  <si>
-    <t>Other</t>
-  </si>
-  <si>
-    <t>Add usage tracking to see how many people finish setup and keep coming back.</t>
-  </si>
-  <si>
-    <t>Before submit (enables L-21)</t>
-  </si>
-  <si>
-    <t>Needed to measure success and the top launch metric.</t>
-  </si>
-  <si>
-    <t>P-4</t>
-  </si>
-  <si>
-    <t>Turn on snap-a-photo receipt scanning and improve how it reads the totals.</t>
-  </si>
-  <si>
-    <t>v1 feature</t>
-  </si>
-  <si>
-    <t>Nearly ready; needs a real device build to switch on and test.</t>
-  </si>
-  <si>
-    <t>P-5</t>
-  </si>
-  <si>
-    <t>Catch bad rows when you import a spreadsheet so imports don't break things.</t>
-  </si>
-  <si>
-    <t>Protects against messy files corrupting your data.</t>
+    <t>P-41</t>
+  </si>
+  <si>
+    <t>Add an 'undo' option after deleting something by mistake.</t>
+  </si>
+  <si>
+    <t>Friendlier than a blocking confirmation pop-up; medium priority.</t>
+  </si>
+  <si>
+    <t>P-39</t>
+  </si>
+  <si>
+    <t>Add loading placeholders and clear offline / syncing states.</t>
+  </si>
+  <si>
+    <t>Makes the app feel smoother while data loads; medium priority.</t>
+  </si>
+  <si>
+    <t>P-34</t>
+  </si>
+  <si>
+    <t>Show how many months your cash savings could cover if income stopped.</t>
+  </si>
+  <si>
+    <t>A reassuring 'safety cushion' number; overlaps the job-loss mode.</t>
+  </si>
+  <si>
+    <t>P-60</t>
+  </si>
+  <si>
+    <t>Let users export their data to a file and import it back.</t>
+  </si>
+  <si>
+    <t>Gives users control of their data; medium priority.</t>
+  </si>
+  <si>
+    <t>V2 — Future</t>
+  </si>
+  <si>
+    <t>EVERYTHING ON THIS TAB IS V2 — a later, bigger release down the road (bank linking, the planning copilot, couples, more retirement modelling, translations, design polish, etc.). If it's not on the V1 or Fast follow-up tabs, it's here. Stage shows how far along each is; 'What's left' spells out what's unfinished for the part-done ones. The yellow 'Your notes' column is yours. To pull anything forward, tell me which tab to move it to. (The crash-reporting row was removed — it's the same work as launch item L-12.)</t>
+  </si>
+  <si>
+    <t>P-1</t>
+  </si>
+  <si>
+    <t>Connect the app to your bank and brokerage so balances and transactions pull in automatically.</t>
+  </si>
+  <si>
+    <t>Biggest convenience and stickiness win, but a large build needing a secure server.</t>
+  </si>
+  <si>
+    <t>P-2</t>
+  </si>
+  <si>
+    <t>Automatically figure out dividends from a stock ticker instead of you typing them in.</t>
+  </si>
+  <si>
+    <t>Saves manual entry for people who hold dividend-paying stocks.</t>
+  </si>
+  <si>
+    <t>P-3</t>
+  </si>
+  <si>
+    <t>Suggest stock tickers as you type and cache prices so they load faster.</t>
+  </si>
+  <si>
+    <t>Nice polish; the core performance views already work.</t>
   </si>
   <si>
     <t>P-6</t>
@@ -585,6 +728,15 @@
     <t>A standout feature that sets the app apart.</t>
   </si>
   <si>
+    <t>P-9</t>
+  </si>
+  <si>
+    <t>Compare life choices like buying a home, having a child, or a job change side by side.</t>
+  </si>
+  <si>
+    <t>Helps users weigh big decisions.</t>
+  </si>
+  <si>
     <t>P-10</t>
   </si>
   <si>
@@ -609,6 +761,24 @@
     <t>Valuable but sensitive; needs careful, accurate tax handling.</t>
   </si>
   <si>
+    <t>P-12</t>
+  </si>
+  <si>
+    <t>Assume your savings grow as your pay rises over the years.</t>
+  </si>
+  <si>
+    <t>Makes retirement projections more realistic.</t>
+  </si>
+  <si>
+    <t>P-13</t>
+  </si>
+  <si>
+    <t>Support married filers and other countries' tax and account rules.</t>
+  </si>
+  <si>
+    <t>Today it only handles single US filers; needed to expand abroad.</t>
+  </si>
+  <si>
     <t>P-14</t>
   </si>
   <si>
@@ -639,6 +809,24 @@
     <t>Fills a life-stage gap many users hit.</t>
   </si>
   <si>
+    <t>P-17</t>
+  </si>
+  <si>
+    <t>Add estate planning like naming who inherits and tracking key documents.</t>
+  </si>
+  <si>
+    <t>Rounds out planning for later life stages.</t>
+  </si>
+  <si>
+    <t>P-18</t>
+  </si>
+  <si>
+    <t>Add a job-loss mode showing how long your cash lasts and a survival budget.</t>
+  </si>
+  <si>
+    <t>Helps people through a stressful transition.</t>
+  </si>
+  <si>
     <t>P-19</t>
   </si>
   <si>
@@ -672,6 +860,42 @@
     <t>Today two logins can't share the same encrypted data; needed for couples.</t>
   </si>
   <si>
+    <t>P-22</t>
+  </si>
+  <si>
+    <t>Add two-step login for stronger account security.</t>
+  </si>
+  <si>
+    <t>App lock already exists; this is the next security layer.</t>
+  </si>
+  <si>
+    <t>P-24</t>
+  </si>
+  <si>
+    <t>Add automated code scanning that flags security flaws as code is written.</t>
+  </si>
+  <si>
+    <t>Catches problems early; lower priority.</t>
+  </si>
+  <si>
+    <t>P-25</t>
+  </si>
+  <si>
+    <t>Scan the finished app file for insecure storage or data-transfer issues.</t>
+  </si>
+  <si>
+    <t>Extra security check; lower priority.</t>
+  </si>
+  <si>
+    <t>P-26</t>
+  </si>
+  <si>
+    <t>Make sure all data fetches use secure, encrypted connections.</t>
+  </si>
+  <si>
+    <t>Protects data in transit; lower priority.</t>
+  </si>
+  <si>
     <t>P-27</t>
   </si>
   <si>
@@ -681,28 +905,31 @@
     <t>App unlock already uses biometrics; this adds per-action confirmation.</t>
   </si>
   <si>
-    <t>P-33</t>
-  </si>
-  <si>
-    <t>UI/UX</t>
-  </si>
-  <si>
-    <t>Add a tap to hide or blur your balances for privacy.</t>
-  </si>
-  <si>
-    <t>Done — verify</t>
-  </si>
-  <si>
-    <t>Lets you check the app in public without showing your money.</t>
-  </si>
-  <si>
-    <t>P-34</t>
-  </si>
-  <si>
-    <t>Show how many months your cash savings could cover if income stopped.</t>
-  </si>
-  <si>
-    <t>A reassuring 'safety cushion' number; overlaps the job-loss mode.</t>
+    <t>P-30</t>
+  </si>
+  <si>
+    <t>Add dark mode and a high-contrast theme.</t>
+  </si>
+  <si>
+    <t>A comfort and readability option; lower priority.</t>
+  </si>
+  <si>
+    <t>P-31</t>
+  </si>
+  <si>
+    <t>Check that all text and charts have enough color contrast to be readable.</t>
+  </si>
+  <si>
+    <t>An accessibility review (for users with disabilities); medium priority.</t>
+  </si>
+  <si>
+    <t>P-32</t>
+  </si>
+  <si>
+    <t>Tone down animations for users who prefer less motion.</t>
+  </si>
+  <si>
+    <t>A small comfort improvement; low priority.</t>
   </si>
   <si>
     <t>P-35</t>
@@ -726,31 +953,22 @@
     <t>Visual consistency across the app.</t>
   </si>
   <si>
-    <t>P-38</t>
-  </si>
-  <si>
-    <t>Make total spending and the category breakdown always add up to the same number.</t>
-  </si>
-  <si>
-    <t>Prevents confusing double-counting between summaries and budget.</t>
-  </si>
-  <si>
-    <t>P-39</t>
-  </si>
-  <si>
-    <t>Add loading placeholders and clear offline / syncing states.</t>
-  </si>
-  <si>
-    <t>Makes the app feel smoother while data loads; medium priority.</t>
-  </si>
-  <si>
-    <t>P-41</t>
-  </si>
-  <si>
-    <t>Add an 'undo' option after deleting something by mistake.</t>
-  </si>
-  <si>
-    <t>Friendlier than a blocking confirmation pop-up; medium priority.</t>
+    <t>P-37</t>
+  </si>
+  <si>
+    <t>Refresh the older detail screens like budget, transactions, settings, and rewards.</t>
+  </si>
+  <si>
+    <t>The new home tiles still open older-looking screens.</t>
+  </si>
+  <si>
+    <t>P-40</t>
+  </si>
+  <si>
+    <t>Add an app-wide banner showing when you're offline or syncing.</t>
+  </si>
+  <si>
+    <t>Keeps users informed about connection status; lower priority.</t>
   </si>
   <si>
     <t>P-42</t>
@@ -774,6 +992,15 @@
     <t>Keeps numbers looking correct and uniform; lower priority.</t>
   </si>
   <si>
+    <t>P-44</t>
+  </si>
+  <si>
+    <t>Let users pin and rearrange the cards on their Home screen.</t>
+  </si>
+  <si>
+    <t>Personalizes the home view; lower priority.</t>
+  </si>
+  <si>
     <t>P-45</t>
   </si>
   <si>
@@ -783,195 +1010,6 @@
     <t>Easier to read for some users; lower priority.</t>
   </si>
   <si>
-    <t>V2 — Future</t>
-  </si>
-  <si>
-    <t>EVERYTHING ON THIS TAB IS V2 (a future release, after the next launch) — grouped by area. There is no in-between: if it's not here, it's in V1. Stage shows how far along each is; 'What's left' spells out what's unfinished for the part-done ones. The yellow 'Your notes' column is yours. To pull any of these INTO the next launch, tell me and I'll move it to the V1 tab. (I removed the crash-reporting row — it's the same work as launch item L-12.)</t>
-  </si>
-  <si>
-    <t>Category</t>
-  </si>
-  <si>
-    <t>What's left</t>
-  </si>
-  <si>
-    <t>Your notes</t>
-  </si>
-  <si>
-    <t>Why it matters</t>
-  </si>
-  <si>
-    <t>P-1</t>
-  </si>
-  <si>
-    <t>Connect the app to your bank and brokerage so balances and transactions pull in automatically.</t>
-  </si>
-  <si>
-    <t>Biggest convenience and stickiness win, but a large build needing a secure server.</t>
-  </si>
-  <si>
-    <t>P-2</t>
-  </si>
-  <si>
-    <t>Automatically figure out dividends from a stock ticker instead of you typing them in.</t>
-  </si>
-  <si>
-    <t>Saves manual entry for people who hold dividend-paying stocks.</t>
-  </si>
-  <si>
-    <t>P-3</t>
-  </si>
-  <si>
-    <t>Suggest stock tickers as you type and cache prices so they load faster.</t>
-  </si>
-  <si>
-    <t>Nice polish; the core performance views already work.</t>
-  </si>
-  <si>
-    <t>P-9</t>
-  </si>
-  <si>
-    <t>Compare life choices like buying a home, having a child, or a job change side by side.</t>
-  </si>
-  <si>
-    <t>Helps users weigh big decisions.</t>
-  </si>
-  <si>
-    <t>P-12</t>
-  </si>
-  <si>
-    <t>Assume your savings grow as your pay rises over the years.</t>
-  </si>
-  <si>
-    <t>Makes retirement projections more realistic.</t>
-  </si>
-  <si>
-    <t>P-13</t>
-  </si>
-  <si>
-    <t>Support married filers and other countries' tax and account rules.</t>
-  </si>
-  <si>
-    <t>Today it only handles single US filers; needed to expand abroad.</t>
-  </si>
-  <si>
-    <t>P-17</t>
-  </si>
-  <si>
-    <t>Add estate planning like naming who inherits and tracking key documents.</t>
-  </si>
-  <si>
-    <t>Rounds out planning for later life stages.</t>
-  </si>
-  <si>
-    <t>P-18</t>
-  </si>
-  <si>
-    <t>Add a job-loss mode showing how long your cash lasts and a survival budget.</t>
-  </si>
-  <si>
-    <t>Helps people through a stressful transition.</t>
-  </si>
-  <si>
-    <t>P-22</t>
-  </si>
-  <si>
-    <t>Add two-step login for stronger account security.</t>
-  </si>
-  <si>
-    <t>App lock already exists; this is the next security layer.</t>
-  </si>
-  <si>
-    <t>P-24</t>
-  </si>
-  <si>
-    <t>Add automated code scanning that flags security flaws as code is written.</t>
-  </si>
-  <si>
-    <t>Catches problems early; lower priority.</t>
-  </si>
-  <si>
-    <t>P-25</t>
-  </si>
-  <si>
-    <t>Scan the finished app file for insecure storage or data-transfer issues.</t>
-  </si>
-  <si>
-    <t>Extra security check; lower priority.</t>
-  </si>
-  <si>
-    <t>P-26</t>
-  </si>
-  <si>
-    <t>Make sure all data fetches use secure, encrypted connections.</t>
-  </si>
-  <si>
-    <t>Protects data in transit; lower priority.</t>
-  </si>
-  <si>
-    <t>P-28</t>
-  </si>
-  <si>
-    <t>Make every screen work with the screen reader for blind and low-vision users.</t>
-  </si>
-  <si>
-    <t>The single biggest accessibility gap (for users with disabilities).</t>
-  </si>
-  <si>
-    <t>P-30</t>
-  </si>
-  <si>
-    <t>Add dark mode and a high-contrast theme.</t>
-  </si>
-  <si>
-    <t>A comfort and readability option; lower priority.</t>
-  </si>
-  <si>
-    <t>P-31</t>
-  </si>
-  <si>
-    <t>Check that all text and charts have enough color contrast to be readable.</t>
-  </si>
-  <si>
-    <t>An accessibility review (for users with disabilities); medium priority.</t>
-  </si>
-  <si>
-    <t>P-32</t>
-  </si>
-  <si>
-    <t>Tone down animations for users who prefer less motion.</t>
-  </si>
-  <si>
-    <t>A small comfort improvement; low priority.</t>
-  </si>
-  <si>
-    <t>P-37</t>
-  </si>
-  <si>
-    <t>Refresh the older detail screens like budget, transactions, settings, and rewards.</t>
-  </si>
-  <si>
-    <t>The new home tiles still open older-looking screens.</t>
-  </si>
-  <si>
-    <t>P-40</t>
-  </si>
-  <si>
-    <t>Add an app-wide banner showing when you're offline or syncing.</t>
-  </si>
-  <si>
-    <t>Keeps users informed about connection status; lower priority.</t>
-  </si>
-  <si>
-    <t>P-44</t>
-  </si>
-  <si>
-    <t>Let users pin and rearrange the cards on their Home screen.</t>
-  </si>
-  <si>
-    <t>Personalizes the home view; lower priority.</t>
-  </si>
-  <si>
     <t>P-46</t>
   </si>
   <si>
@@ -1029,9 +1067,6 @@
     <t>P-52</t>
   </si>
   <si>
-    <t>Growth</t>
-  </si>
-  <si>
     <t>Send reminder nudges like 'you're near your dining budget'.</t>
   </si>
   <si>
@@ -1041,18 +1076,6 @@
     <t>Drives people back into the app.</t>
   </si>
   <si>
-    <t>P-53</t>
-  </si>
-  <si>
-    <t>Finish the full savings-goals screen with progress, priority, and projections.</t>
-  </si>
-  <si>
-    <t>The goals tab and funding logic exist; the full visual screen isn't finished.</t>
-  </si>
-  <si>
-    <t>Helps people set and track goals; a stickiness feature.</t>
-  </si>
-  <si>
     <t>P-54</t>
   </si>
   <si>
@@ -1101,15 +1124,6 @@
     <t>Ensures numbers look right everywhere.</t>
   </si>
   <si>
-    <t>P-60</t>
-  </si>
-  <si>
-    <t>Let users export their data to a file and import it back.</t>
-  </si>
-  <si>
-    <t>Gives users control of their data; medium priority.</t>
-  </si>
-  <si>
     <t>P-61</t>
   </si>
   <si>
@@ -1117,15 +1131,6 @@
   </si>
   <si>
     <t>Prevents data problems when the app updates.</t>
-  </si>
-  <si>
-    <t>P-62</t>
-  </si>
-  <si>
-    <t>Add tests for the core retirement and investment math.</t>
-  </si>
-  <si>
-    <t>Protects accuracy of the most important calculations; high priority.</t>
   </si>
   <si>
     <t>P-65</t>
@@ -1671,7 +1676,7 @@
   <sheetPr>
     <tabColor rgb="FFC00000"/>
   </sheetPr>
-  <dimension ref="A1:L60"/>
+  <dimension ref="A1:L34"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="6.7109375" customWidth="1"/>
@@ -2825,858 +2830,26 @@
         <v>26</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="F34" s="5" t="s">
-        <v>19</v>
+        <v>161</v>
+      </c>
+      <c r="F34" s="8" t="s">
+        <v>35</v>
       </c>
       <c r="G34" s="4" t="s">
-        <v>147</v>
+        <v>162</v>
       </c>
       <c r="H34" s="6"/>
       <c r="I34" s="6"/>
       <c r="J34" s="6"/>
       <c r="K34" s="6" t="s">
-        <v>152</v>
+        <v>37</v>
       </c>
       <c r="L34" s="4" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="35" spans="1:12">
-      <c r="A35" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="C35" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="D35" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E35" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="F35" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G35" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="H35" s="6"/>
-      <c r="I35" s="6"/>
-      <c r="J35" s="6"/>
-      <c r="K35" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="L35" s="4" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="36" spans="1:12">
-      <c r="A36" s="4" t="s">
-        <v>165</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>167</v>
-      </c>
-      <c r="D36" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E36" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="F36" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G36" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="H36" s="6"/>
-      <c r="I36" s="6"/>
-      <c r="J36" s="6"/>
-      <c r="K36" s="6" t="s">
-        <v>168</v>
-      </c>
-      <c r="L36" s="4" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="37" spans="1:12">
-      <c r="A37" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="D37" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E37" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="F37" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G37" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="H37" s="6"/>
-      <c r="I37" s="6"/>
-      <c r="J37" s="6"/>
-      <c r="K37" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="L37" s="4" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="38" spans="1:12">
-      <c r="A38" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="B38" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C38" s="4" t="s">
-        <v>175</v>
-      </c>
-      <c r="D38" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E38" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="F38" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G38" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="H38" s="6"/>
-      <c r="I38" s="6"/>
-      <c r="J38" s="6"/>
-      <c r="K38" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="L38" s="4" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="39" spans="1:12">
-      <c r="A39" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="B39" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="C39" s="4" t="s">
-        <v>179</v>
-      </c>
-      <c r="D39" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E39" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="F39" s="10" t="s">
-        <v>76</v>
-      </c>
-      <c r="G39" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="H39" s="6"/>
-      <c r="I39" s="6"/>
-      <c r="J39" s="6"/>
-      <c r="K39" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="L39" s="4" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="40" spans="1:12">
-      <c r="A40" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="B40" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="C40" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="D40" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E40" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="F40" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G40" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="H40" s="6"/>
-      <c r="I40" s="6"/>
-      <c r="J40" s="6"/>
-      <c r="K40" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="L40" s="4" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="41" spans="1:12">
-      <c r="A41" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="B41" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="C41" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="D41" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E41" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="F41" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G41" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="H41" s="6"/>
-      <c r="I41" s="6"/>
-      <c r="J41" s="6"/>
-      <c r="K41" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="L41" s="4" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="42" spans="1:12">
-      <c r="A42" s="4" t="s">
-        <v>188</v>
-      </c>
-      <c r="B42" s="4" t="s">
-        <v>189</v>
-      </c>
-      <c r="C42" s="4" t="s">
-        <v>190</v>
-      </c>
-      <c r="D42" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E42" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="F42" s="10" t="s">
-        <v>76</v>
-      </c>
-      <c r="G42" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="H42" s="6"/>
-      <c r="I42" s="6"/>
-      <c r="J42" s="6"/>
-      <c r="K42" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="L42" s="4" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="43" spans="1:12">
-      <c r="A43" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="B43" s="4" t="s">
-        <v>189</v>
-      </c>
-      <c r="C43" s="4" t="s">
-        <v>194</v>
-      </c>
-      <c r="D43" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E43" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="F43" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G43" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="H43" s="6"/>
-      <c r="I43" s="6"/>
-      <c r="J43" s="6"/>
-      <c r="K43" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="L43" s="4" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="44" spans="1:12">
-      <c r="A44" s="4" t="s">
-        <v>196</v>
-      </c>
-      <c r="B44" s="4" t="s">
-        <v>189</v>
-      </c>
-      <c r="C44" s="4" t="s">
-        <v>197</v>
-      </c>
-      <c r="D44" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E44" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="F44" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G44" s="4" t="s">
-        <v>198</v>
-      </c>
-      <c r="H44" s="6"/>
-      <c r="I44" s="6"/>
-      <c r="J44" s="6"/>
-      <c r="K44" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="L44" s="4" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="45" spans="1:12">
-      <c r="A45" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="B45" s="4" t="s">
-        <v>189</v>
-      </c>
-      <c r="C45" s="4" t="s">
-        <v>201</v>
-      </c>
-      <c r="D45" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E45" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="F45" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G45" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="H45" s="6"/>
-      <c r="I45" s="6"/>
-      <c r="J45" s="6"/>
-      <c r="K45" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="L45" s="4" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="46" spans="1:12">
-      <c r="A46" s="4" t="s">
-        <v>203</v>
-      </c>
-      <c r="B46" s="4" t="s">
-        <v>189</v>
-      </c>
-      <c r="C46" s="4" t="s">
-        <v>204</v>
-      </c>
-      <c r="D46" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E46" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="F46" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G46" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="H46" s="6"/>
-      <c r="I46" s="6"/>
-      <c r="J46" s="6"/>
-      <c r="K46" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="L46" s="4" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="47" spans="1:12">
-      <c r="A47" s="4" t="s">
-        <v>206</v>
-      </c>
-      <c r="B47" s="4" t="s">
-        <v>189</v>
-      </c>
-      <c r="C47" s="4" t="s">
-        <v>207</v>
-      </c>
-      <c r="D47" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E47" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="F47" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G47" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="H47" s="6"/>
-      <c r="I47" s="6"/>
-      <c r="J47" s="6"/>
-      <c r="K47" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="L47" s="4" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="48" spans="1:12">
-      <c r="A48" s="4" t="s">
-        <v>209</v>
-      </c>
-      <c r="B48" s="4" t="s">
-        <v>210</v>
-      </c>
-      <c r="C48" s="4" t="s">
-        <v>211</v>
-      </c>
-      <c r="D48" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E48" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="F48" s="10" t="s">
-        <v>76</v>
-      </c>
-      <c r="G48" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="H48" s="6"/>
-      <c r="I48" s="6"/>
-      <c r="J48" s="6"/>
-      <c r="K48" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="L48" s="4" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="49" spans="1:12">
-      <c r="A49" s="4" t="s">
-        <v>214</v>
-      </c>
-      <c r="B49" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="C49" s="4" t="s">
-        <v>215</v>
-      </c>
-      <c r="D49" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E49" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="F49" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G49" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="H49" s="6"/>
-      <c r="I49" s="6"/>
-      <c r="J49" s="6"/>
-      <c r="K49" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="L49" s="4" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="50" spans="1:12">
-      <c r="A50" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="B50" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="C50" s="4" t="s">
-        <v>218</v>
-      </c>
-      <c r="D50" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E50" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="F50" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G50" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="H50" s="6"/>
-      <c r="I50" s="6"/>
-      <c r="J50" s="6"/>
-      <c r="K50" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="L50" s="4" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="51" spans="1:12">
-      <c r="A51" s="4" t="s">
-        <v>220</v>
-      </c>
-      <c r="B51" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="C51" s="4" t="s">
-        <v>222</v>
-      </c>
-      <c r="D51" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E51" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="F51" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="G51" s="4" t="s">
-        <v>223</v>
-      </c>
-      <c r="H51" s="6"/>
-      <c r="I51" s="6"/>
-      <c r="J51" s="6"/>
-      <c r="K51" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="L51" s="4" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="52" spans="1:12">
-      <c r="A52" s="4" t="s">
-        <v>225</v>
-      </c>
-      <c r="B52" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="C52" s="4" t="s">
-        <v>226</v>
-      </c>
-      <c r="D52" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E52" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="F52" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G52" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="H52" s="6"/>
-      <c r="I52" s="6"/>
-      <c r="J52" s="6"/>
-      <c r="K52" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="L52" s="4" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="53" spans="1:12">
-      <c r="A53" s="4" t="s">
-        <v>228</v>
-      </c>
-      <c r="B53" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="C53" s="4" t="s">
-        <v>229</v>
-      </c>
-      <c r="D53" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E53" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="F53" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G53" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="H53" s="6"/>
-      <c r="I53" s="6"/>
-      <c r="J53" s="6"/>
-      <c r="K53" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="L53" s="4" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="54" spans="1:12">
-      <c r="A54" s="4" t="s">
-        <v>231</v>
-      </c>
-      <c r="B54" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="C54" s="4" t="s">
-        <v>232</v>
-      </c>
-      <c r="D54" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E54" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="F54" s="10" t="s">
-        <v>76</v>
-      </c>
-      <c r="G54" s="4" t="s">
-        <v>233</v>
-      </c>
-      <c r="H54" s="6"/>
-      <c r="I54" s="6"/>
-      <c r="J54" s="6"/>
-      <c r="K54" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="L54" s="4" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="55" spans="1:12">
-      <c r="A55" s="4" t="s">
-        <v>235</v>
-      </c>
-      <c r="B55" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="C55" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="D55" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E55" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="F55" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G55" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="H55" s="6"/>
-      <c r="I55" s="6"/>
-      <c r="J55" s="6"/>
-      <c r="K55" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="L55" s="4" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="56" spans="1:12">
-      <c r="A56" s="4" t="s">
-        <v>238</v>
-      </c>
-      <c r="B56" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="C56" s="4" t="s">
-        <v>239</v>
-      </c>
-      <c r="D56" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E56" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="F56" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G56" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="H56" s="6"/>
-      <c r="I56" s="6"/>
-      <c r="J56" s="6"/>
-      <c r="K56" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="L56" s="4" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="57" spans="1:12">
-      <c r="A57" s="4" t="s">
-        <v>241</v>
-      </c>
-      <c r="B57" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="C57" s="4" t="s">
-        <v>242</v>
-      </c>
-      <c r="D57" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E57" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="F57" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G57" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="H57" s="6"/>
-      <c r="I57" s="6"/>
-      <c r="J57" s="6"/>
-      <c r="K57" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="L57" s="4" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="58" spans="1:12">
-      <c r="A58" s="4" t="s">
-        <v>244</v>
-      </c>
-      <c r="B58" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="C58" s="4" t="s">
-        <v>245</v>
-      </c>
-      <c r="D58" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E58" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="F58" s="10" t="s">
-        <v>76</v>
-      </c>
-      <c r="G58" s="4" t="s">
-        <v>246</v>
-      </c>
-      <c r="H58" s="6"/>
-      <c r="I58" s="6"/>
-      <c r="J58" s="6"/>
-      <c r="K58" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="L58" s="4" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="59" spans="1:12">
-      <c r="A59" s="4" t="s">
-        <v>248</v>
-      </c>
-      <c r="B59" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="C59" s="4" t="s">
-        <v>249</v>
-      </c>
-      <c r="D59" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E59" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="F59" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G59" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="H59" s="6"/>
-      <c r="I59" s="6"/>
-      <c r="J59" s="6"/>
-      <c r="K59" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="L59" s="4" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="60" spans="1:12">
-      <c r="A60" s="4" t="s">
-        <v>251</v>
-      </c>
-      <c r="B60" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="C60" s="4" t="s">
-        <v>252</v>
-      </c>
-      <c r="D60" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E60" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="F60" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G60" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="H60" s="6"/>
-      <c r="I60" s="6"/>
-      <c r="J60" s="6"/>
-      <c r="K60" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="L60" s="4" t="s">
-        <v>253</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:L60"/>
+  <autoFilter ref="A4:L34"/>
   <mergeCells count="2">
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:L3"/>
@@ -3688,9 +2861,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
-    <tabColor rgb="FF1F4E5F"/>
+    <tabColor rgb="FFE69138"/>
   </sheetPr>
-  <dimension ref="A1:G47"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="6.7109375" customWidth="1"/>
@@ -3704,7 +2877,7 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>254</v>
+        <v>164</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3715,7 +2888,7 @@
     </row>
     <row r="2" spans="1:7" ht="28" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>255</v>
+        <v>165</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3738,7 +2911,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>256</v>
+        <v>166</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>4</v>
@@ -3747,24 +2920,24 @@
         <v>7</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>257</v>
+        <v>167</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>258</v>
+        <v>168</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>259</v>
+        <v>169</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="4" t="s">
-        <v>260</v>
+        <v>170</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>15</v>
+        <v>155</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>261</v>
+        <v>171</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>19</v>
@@ -3772,18 +2945,18 @@
       <c r="E5" s="4"/>
       <c r="F5" s="6"/>
       <c r="G5" s="4" t="s">
-        <v>262</v>
+        <v>172</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="4" t="s">
-        <v>263</v>
+        <v>173</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>15</v>
+        <v>159</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>264</v>
+        <v>174</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>19</v>
@@ -3791,18 +2964,18 @@
       <c r="E6" s="4"/>
       <c r="F6" s="6"/>
       <c r="G6" s="4" t="s">
-        <v>265</v>
+        <v>175</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="4" t="s">
-        <v>266</v>
+        <v>176</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>15</v>
+        <v>155</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>267</v>
+        <v>177</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>19</v>
@@ -3810,18 +2983,18 @@
       <c r="E7" s="4"/>
       <c r="F7" s="6"/>
       <c r="G7" s="4" t="s">
-        <v>268</v>
+        <v>178</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="4" t="s">
-        <v>269</v>
+        <v>179</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>270</v>
+        <v>181</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>19</v>
@@ -3829,18 +3002,18 @@
       <c r="E8" s="4"/>
       <c r="F8" s="6"/>
       <c r="G8" s="4" t="s">
-        <v>271</v>
+        <v>182</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="4" t="s">
-        <v>272</v>
+        <v>183</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>189</v>
+        <v>15</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>273</v>
+        <v>184</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>19</v>
@@ -3848,18 +3021,18 @@
       <c r="E9" s="4"/>
       <c r="F9" s="6"/>
       <c r="G9" s="4" t="s">
-        <v>274</v>
+        <v>185</v>
       </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="4" t="s">
-        <v>275</v>
+        <v>186</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>189</v>
+        <v>15</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>276</v>
+        <v>187</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>19</v>
@@ -3867,18 +3040,350 @@
       <c r="E10" s="4"/>
       <c r="F10" s="6"/>
       <c r="G10" s="4" t="s">
-        <v>277</v>
+        <v>188</v>
       </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" s="4" t="s">
-        <v>278</v>
+        <v>189</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>279</v>
+        <v>191</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="F11" s="6"/>
+      <c r="G11" s="4" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" s="4"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="4" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E13" s="4"/>
+      <c r="F13" s="6"/>
+      <c r="G13" s="4" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E14" s="4"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="4" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E15" s="4"/>
+      <c r="F15" s="6"/>
+      <c r="G15" s="4" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E16" s="4"/>
+      <c r="F16" s="6"/>
+      <c r="G16" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E17" s="4"/>
+      <c r="F17" s="6"/>
+      <c r="G17" s="4" t="s">
+        <v>212</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:G17"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <tabColor rgb="FF1F4E5F"/>
+  </sheetPr>
+  <dimension ref="A1:G60"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="6.7109375" customWidth="1"/>
+    <col min="2" max="2" width="13.7109375" customWidth="1"/>
+    <col min="3" max="3" width="52.7109375" customWidth="1"/>
+    <col min="4" max="4" width="8.7109375" customWidth="1"/>
+    <col min="5" max="5" width="34.7109375" customWidth="1"/>
+    <col min="6" max="6" width="18.7109375" customWidth="1"/>
+    <col min="7" max="7" width="52.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+    </row>
+    <row r="2" spans="1:7" ht="28" customHeight="1">
+      <c r="A2" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+    </row>
+    <row r="4" spans="1:7" ht="30" customHeight="1">
+      <c r="A4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="4"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="4" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" s="4"/>
+      <c r="F6" s="6"/>
+      <c r="G6" s="4" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" s="4"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="4" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="F8" s="6"/>
+      <c r="G8" s="4" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>230</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E9" s="4"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="4" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" s="4"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="4" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>236</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>19</v>
@@ -3886,37 +3391,39 @@
       <c r="E11" s="4"/>
       <c r="F11" s="6"/>
       <c r="G11" s="4" t="s">
-        <v>280</v>
+        <v>237</v>
       </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="4" t="s">
-        <v>281</v>
+        <v>238</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>189</v>
+        <v>239</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>282</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E12" s="4"/>
+        <v>240</v>
+      </c>
+      <c r="D12" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>241</v>
+      </c>
       <c r="F12" s="6"/>
       <c r="G12" s="4" t="s">
-        <v>283</v>
+        <v>242</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" s="4" t="s">
-        <v>284</v>
+        <v>243</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>45</v>
+        <v>239</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>285</v>
+        <v>244</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>19</v>
@@ -3924,18 +3431,18 @@
       <c r="E13" s="4"/>
       <c r="F13" s="6"/>
       <c r="G13" s="4" t="s">
-        <v>286</v>
+        <v>245</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="4" t="s">
-        <v>287</v>
+        <v>246</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>45</v>
+        <v>239</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>288</v>
+        <v>247</v>
       </c>
       <c r="D14" s="5" t="s">
         <v>19</v>
@@ -3943,18 +3450,18 @@
       <c r="E14" s="4"/>
       <c r="F14" s="6"/>
       <c r="G14" s="4" t="s">
-        <v>289</v>
+        <v>248</v>
       </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" s="4" t="s">
-        <v>290</v>
+        <v>249</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>45</v>
+        <v>239</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>291</v>
+        <v>250</v>
       </c>
       <c r="D15" s="5" t="s">
         <v>19</v>
@@ -3962,37 +3469,39 @@
       <c r="E15" s="4"/>
       <c r="F15" s="6"/>
       <c r="G15" s="4" t="s">
-        <v>292</v>
+        <v>251</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="4" t="s">
-        <v>293</v>
+        <v>252</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>45</v>
+        <v>239</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>294</v>
+        <v>253</v>
       </c>
       <c r="D16" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="E16" s="4"/>
+      <c r="E16" s="4" t="s">
+        <v>254</v>
+      </c>
       <c r="F16" s="6"/>
       <c r="G16" s="4" t="s">
-        <v>295</v>
+        <v>255</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="4" t="s">
-        <v>296</v>
+        <v>256</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>155</v>
+        <v>239</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>297</v>
+        <v>257</v>
       </c>
       <c r="D17" s="5" t="s">
         <v>19</v>
@@ -4000,18 +3509,18 @@
       <c r="E17" s="4"/>
       <c r="F17" s="6"/>
       <c r="G17" s="4" t="s">
-        <v>298</v>
+        <v>258</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" s="4" t="s">
-        <v>299</v>
+        <v>259</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>155</v>
+        <v>239</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>300</v>
+        <v>260</v>
       </c>
       <c r="D18" s="5" t="s">
         <v>19</v>
@@ -4019,18 +3528,18 @@
       <c r="E18" s="4"/>
       <c r="F18" s="6"/>
       <c r="G18" s="4" t="s">
-        <v>301</v>
+        <v>261</v>
       </c>
     </row>
     <row r="19" spans="1:7">
       <c r="A19" s="4" t="s">
-        <v>302</v>
+        <v>262</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>155</v>
+        <v>239</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>303</v>
+        <v>263</v>
       </c>
       <c r="D19" s="5" t="s">
         <v>19</v>
@@ -4038,18 +3547,18 @@
       <c r="E19" s="4"/>
       <c r="F19" s="6"/>
       <c r="G19" s="4" t="s">
-        <v>304</v>
+        <v>264</v>
       </c>
     </row>
     <row r="20" spans="1:7">
       <c r="A20" s="4" t="s">
-        <v>305</v>
+        <v>265</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>155</v>
+        <v>239</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>306</v>
+        <v>266</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>19</v>
@@ -4057,18 +3566,18 @@
       <c r="E20" s="4"/>
       <c r="F20" s="6"/>
       <c r="G20" s="4" t="s">
-        <v>307</v>
+        <v>267</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="4" t="s">
-        <v>308</v>
+        <v>268</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>221</v>
+        <v>239</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>309</v>
+        <v>269</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>19</v>
@@ -4076,37 +3585,39 @@
       <c r="E21" s="4"/>
       <c r="F21" s="6"/>
       <c r="G21" s="4" t="s">
-        <v>310</v>
+        <v>270</v>
       </c>
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="4" t="s">
-        <v>311</v>
+        <v>271</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>221</v>
+        <v>272</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>312</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E22" s="4"/>
+        <v>273</v>
+      </c>
+      <c r="D22" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>274</v>
+      </c>
       <c r="F22" s="6"/>
       <c r="G22" s="4" t="s">
-        <v>313</v>
+        <v>275</v>
       </c>
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="4" t="s">
-        <v>314</v>
+        <v>276</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>221</v>
+        <v>45</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>315</v>
+        <v>277</v>
       </c>
       <c r="D23" s="5" t="s">
         <v>19</v>
@@ -4114,18 +3625,18 @@
       <c r="E23" s="4"/>
       <c r="F23" s="6"/>
       <c r="G23" s="4" t="s">
-        <v>316</v>
+        <v>278</v>
       </c>
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="4" t="s">
-        <v>317</v>
+        <v>279</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>221</v>
+        <v>45</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>318</v>
+        <v>280</v>
       </c>
       <c r="D24" s="5" t="s">
         <v>19</v>
@@ -4133,18 +3644,18 @@
       <c r="E24" s="4"/>
       <c r="F24" s="6"/>
       <c r="G24" s="4" t="s">
-        <v>319</v>
+        <v>281</v>
       </c>
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="4" t="s">
-        <v>320</v>
+        <v>282</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>221</v>
+        <v>45</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>321</v>
+        <v>283</v>
       </c>
       <c r="D25" s="5" t="s">
         <v>19</v>
@@ -4152,18 +3663,18 @@
       <c r="E25" s="4"/>
       <c r="F25" s="6"/>
       <c r="G25" s="4" t="s">
-        <v>322</v>
+        <v>284</v>
       </c>
     </row>
     <row r="26" spans="1:7">
       <c r="A26" s="4" t="s">
-        <v>323</v>
+        <v>285</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>221</v>
+        <v>45</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>324</v>
+        <v>286</v>
       </c>
       <c r="D26" s="5" t="s">
         <v>19</v>
@@ -4171,18 +3682,18 @@
       <c r="E26" s="4"/>
       <c r="F26" s="6"/>
       <c r="G26" s="4" t="s">
-        <v>325</v>
+        <v>287</v>
       </c>
     </row>
     <row r="27" spans="1:7">
       <c r="A27" s="4" t="s">
-        <v>326</v>
+        <v>288</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>221</v>
+        <v>45</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>327</v>
+        <v>289</v>
       </c>
       <c r="D27" s="5" t="s">
         <v>19</v>
@@ -4190,18 +3701,18 @@
       <c r="E27" s="4"/>
       <c r="F27" s="6"/>
       <c r="G27" s="4" t="s">
-        <v>328</v>
+        <v>290</v>
       </c>
     </row>
     <row r="28" spans="1:7">
       <c r="A28" s="4" t="s">
-        <v>329</v>
+        <v>291</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>221</v>
+        <v>45</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>330</v>
+        <v>292</v>
       </c>
       <c r="D28" s="5" t="s">
         <v>19</v>
@@ -4209,18 +3720,18 @@
       <c r="E28" s="4"/>
       <c r="F28" s="6"/>
       <c r="G28" s="4" t="s">
-        <v>331</v>
+        <v>293</v>
       </c>
     </row>
     <row r="29" spans="1:7">
       <c r="A29" s="4" t="s">
-        <v>332</v>
+        <v>294</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>221</v>
+        <v>195</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>333</v>
+        <v>295</v>
       </c>
       <c r="D29" s="5" t="s">
         <v>19</v>
@@ -4228,60 +3739,56 @@
       <c r="E29" s="4"/>
       <c r="F29" s="6"/>
       <c r="G29" s="4" t="s">
-        <v>334</v>
+        <v>296</v>
       </c>
     </row>
     <row r="30" spans="1:7">
       <c r="A30" s="4" t="s">
-        <v>335</v>
+        <v>297</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>336</v>
+        <v>195</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>337</v>
+        <v>298</v>
       </c>
       <c r="D30" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="E30" s="4" t="s">
-        <v>338</v>
-      </c>
+      <c r="E30" s="4"/>
       <c r="F30" s="6"/>
       <c r="G30" s="4" t="s">
-        <v>339</v>
+        <v>299</v>
       </c>
     </row>
     <row r="31" spans="1:7">
       <c r="A31" s="4" t="s">
-        <v>340</v>
+        <v>300</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>336</v>
+        <v>195</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>341</v>
-      </c>
-      <c r="D31" s="10" t="s">
-        <v>76</v>
-      </c>
-      <c r="E31" s="4" t="s">
-        <v>342</v>
-      </c>
+        <v>301</v>
+      </c>
+      <c r="D31" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E31" s="4"/>
       <c r="F31" s="6"/>
       <c r="G31" s="4" t="s">
-        <v>343</v>
+        <v>302</v>
       </c>
     </row>
     <row r="32" spans="1:7">
       <c r="A32" s="4" t="s">
-        <v>344</v>
+        <v>303</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>336</v>
+        <v>159</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>345</v>
+        <v>304</v>
       </c>
       <c r="D32" s="5" t="s">
         <v>19</v>
@@ -4289,37 +3796,39 @@
       <c r="E32" s="4"/>
       <c r="F32" s="6"/>
       <c r="G32" s="4" t="s">
-        <v>346</v>
+        <v>305</v>
       </c>
     </row>
     <row r="33" spans="1:7">
       <c r="A33" s="4" t="s">
-        <v>347</v>
+        <v>306</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>336</v>
+        <v>159</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>348</v>
-      </c>
-      <c r="D33" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E33" s="4"/>
+        <v>307</v>
+      </c>
+      <c r="D33" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>308</v>
+      </c>
       <c r="F33" s="6"/>
       <c r="G33" s="4" t="s">
-        <v>349</v>
+        <v>309</v>
       </c>
     </row>
     <row r="34" spans="1:7">
       <c r="A34" s="4" t="s">
-        <v>350</v>
+        <v>310</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>336</v>
+        <v>159</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>351</v>
+        <v>311</v>
       </c>
       <c r="D34" s="5" t="s">
         <v>19</v>
@@ -4327,18 +3836,18 @@
       <c r="E34" s="4"/>
       <c r="F34" s="6"/>
       <c r="G34" s="4" t="s">
-        <v>352</v>
+        <v>312</v>
       </c>
     </row>
     <row r="35" spans="1:7">
       <c r="A35" s="4" t="s">
-        <v>353</v>
+        <v>313</v>
       </c>
       <c r="B35" s="4" t="s">
         <v>159</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>354</v>
+        <v>314</v>
       </c>
       <c r="D35" s="5" t="s">
         <v>19</v>
@@ -4346,39 +3855,39 @@
       <c r="E35" s="4"/>
       <c r="F35" s="6"/>
       <c r="G35" s="4" t="s">
-        <v>355</v>
+        <v>315</v>
       </c>
     </row>
     <row r="36" spans="1:7">
       <c r="A36" s="4" t="s">
-        <v>356</v>
+        <v>316</v>
       </c>
       <c r="B36" s="4" t="s">
         <v>159</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>357</v>
+        <v>317</v>
       </c>
       <c r="D36" s="10" t="s">
         <v>76</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>358</v>
+        <v>318</v>
       </c>
       <c r="F36" s="6"/>
       <c r="G36" s="4" t="s">
-        <v>359</v>
+        <v>319</v>
       </c>
     </row>
     <row r="37" spans="1:7">
       <c r="A37" s="4" t="s">
-        <v>360</v>
+        <v>320</v>
       </c>
       <c r="B37" s="4" t="s">
         <v>159</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>361</v>
+        <v>321</v>
       </c>
       <c r="D37" s="5" t="s">
         <v>19</v>
@@ -4386,18 +3895,18 @@
       <c r="E37" s="4"/>
       <c r="F37" s="6"/>
       <c r="G37" s="4" t="s">
-        <v>362</v>
+        <v>322</v>
       </c>
     </row>
     <row r="38" spans="1:7">
       <c r="A38" s="4" t="s">
-        <v>363</v>
+        <v>323</v>
       </c>
       <c r="B38" s="4" t="s">
         <v>159</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>364</v>
+        <v>324</v>
       </c>
       <c r="D38" s="5" t="s">
         <v>19</v>
@@ -4405,18 +3914,18 @@
       <c r="E38" s="4"/>
       <c r="F38" s="6"/>
       <c r="G38" s="4" t="s">
-        <v>365</v>
+        <v>325</v>
       </c>
     </row>
     <row r="39" spans="1:7">
       <c r="A39" s="4" t="s">
-        <v>366</v>
+        <v>326</v>
       </c>
       <c r="B39" s="4" t="s">
         <v>159</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>367</v>
+        <v>327</v>
       </c>
       <c r="D39" s="5" t="s">
         <v>19</v>
@@ -4424,18 +3933,18 @@
       <c r="E39" s="4"/>
       <c r="F39" s="6"/>
       <c r="G39" s="4" t="s">
-        <v>368</v>
+        <v>328</v>
       </c>
     </row>
     <row r="40" spans="1:7">
       <c r="A40" s="4" t="s">
-        <v>369</v>
+        <v>329</v>
       </c>
       <c r="B40" s="4" t="s">
         <v>159</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>370</v>
+        <v>330</v>
       </c>
       <c r="D40" s="5" t="s">
         <v>19</v>
@@ -4443,18 +3952,18 @@
       <c r="E40" s="4"/>
       <c r="F40" s="6"/>
       <c r="G40" s="4" t="s">
-        <v>371</v>
+        <v>331</v>
       </c>
     </row>
     <row r="41" spans="1:7">
       <c r="A41" s="4" t="s">
-        <v>372</v>
+        <v>332</v>
       </c>
       <c r="B41" s="4" t="s">
         <v>159</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>373</v>
+        <v>333</v>
       </c>
       <c r="D41" s="5" t="s">
         <v>19</v>
@@ -4462,18 +3971,18 @@
       <c r="E41" s="4"/>
       <c r="F41" s="6"/>
       <c r="G41" s="4" t="s">
-        <v>374</v>
+        <v>334</v>
       </c>
     </row>
     <row r="42" spans="1:7">
       <c r="A42" s="4" t="s">
-        <v>375</v>
+        <v>335</v>
       </c>
       <c r="B42" s="4" t="s">
         <v>159</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>376</v>
+        <v>336</v>
       </c>
       <c r="D42" s="5" t="s">
         <v>19</v>
@@ -4481,18 +3990,18 @@
       <c r="E42" s="4"/>
       <c r="F42" s="6"/>
       <c r="G42" s="4" t="s">
-        <v>377</v>
+        <v>337</v>
       </c>
     </row>
     <row r="43" spans="1:7">
       <c r="A43" s="4" t="s">
-        <v>378</v>
+        <v>338</v>
       </c>
       <c r="B43" s="4" t="s">
         <v>159</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>379</v>
+        <v>339</v>
       </c>
       <c r="D43" s="5" t="s">
         <v>19</v>
@@ -4500,18 +4009,18 @@
       <c r="E43" s="4"/>
       <c r="F43" s="6"/>
       <c r="G43" s="4" t="s">
-        <v>380</v>
+        <v>340</v>
       </c>
     </row>
     <row r="44" spans="1:7">
       <c r="A44" s="4" t="s">
-        <v>381</v>
+        <v>341</v>
       </c>
       <c r="B44" s="4" t="s">
         <v>159</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>382</v>
+        <v>342</v>
       </c>
       <c r="D44" s="5" t="s">
         <v>19</v>
@@ -4519,18 +4028,18 @@
       <c r="E44" s="4"/>
       <c r="F44" s="6"/>
       <c r="G44" s="4" t="s">
-        <v>383</v>
+        <v>343</v>
       </c>
     </row>
     <row r="45" spans="1:7">
       <c r="A45" s="4" t="s">
-        <v>384</v>
+        <v>344</v>
       </c>
       <c r="B45" s="4" t="s">
         <v>159</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>385</v>
+        <v>345</v>
       </c>
       <c r="D45" s="5" t="s">
         <v>19</v>
@@ -4538,37 +4047,39 @@
       <c r="E45" s="4"/>
       <c r="F45" s="6"/>
       <c r="G45" s="4" t="s">
-        <v>386</v>
+        <v>346</v>
       </c>
     </row>
     <row r="46" spans="1:7">
       <c r="A46" s="4" t="s">
-        <v>387</v>
+        <v>347</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>166</v>
+        <v>190</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>388</v>
+        <v>348</v>
       </c>
       <c r="D46" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="E46" s="4"/>
+      <c r="E46" s="4" t="s">
+        <v>349</v>
+      </c>
       <c r="F46" s="6"/>
       <c r="G46" s="4" t="s">
-        <v>389</v>
+        <v>350</v>
       </c>
     </row>
     <row r="47" spans="1:7">
       <c r="A47" s="4" t="s">
-        <v>390</v>
+        <v>351</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>166</v>
+        <v>190</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>391</v>
+        <v>352</v>
       </c>
       <c r="D47" s="5" t="s">
         <v>19</v>
@@ -4576,11 +4087,260 @@
       <c r="E47" s="4"/>
       <c r="F47" s="6"/>
       <c r="G47" s="4" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7">
+      <c r="A48" s="4" t="s">
+        <v>354</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>355</v>
+      </c>
+      <c r="D48" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E48" s="4"/>
+      <c r="F48" s="6"/>
+      <c r="G48" s="4" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7">
+      <c r="A49" s="4" t="s">
+        <v>357</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>358</v>
+      </c>
+      <c r="D49" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E49" s="4"/>
+      <c r="F49" s="6"/>
+      <c r="G49" s="4" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7">
+      <c r="A50" s="4" t="s">
+        <v>360</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>361</v>
+      </c>
+      <c r="D50" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E50" s="4"/>
+      <c r="F50" s="6"/>
+      <c r="G50" s="4" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7">
+      <c r="A51" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>364</v>
+      </c>
+      <c r="D51" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="E51" s="4" t="s">
+        <v>365</v>
+      </c>
+      <c r="F51" s="6"/>
+      <c r="G51" s="4" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7">
+      <c r="A52" s="4" t="s">
+        <v>367</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>368</v>
+      </c>
+      <c r="D52" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E52" s="4"/>
+      <c r="F52" s="6"/>
+      <c r="G52" s="4" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7">
+      <c r="A53" s="4" t="s">
+        <v>370</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="D53" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E53" s="4"/>
+      <c r="F53" s="6"/>
+      <c r="G53" s="4" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7">
+      <c r="A54" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>374</v>
+      </c>
+      <c r="D54" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E54" s="4"/>
+      <c r="F54" s="6"/>
+      <c r="G54" s="4" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7">
+      <c r="A55" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="D55" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E55" s="4"/>
+      <c r="F55" s="6"/>
+      <c r="G55" s="4" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7">
+      <c r="A56" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>380</v>
+      </c>
+      <c r="D56" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E56" s="4"/>
+      <c r="F56" s="6"/>
+      <c r="G56" s="4" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7">
+      <c r="A57" s="4" t="s">
+        <v>382</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>383</v>
+      </c>
+      <c r="D57" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E57" s="4"/>
+      <c r="F57" s="6"/>
+      <c r="G57" s="4" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7">
+      <c r="A58" s="4" t="s">
+        <v>385</v>
+      </c>
+      <c r="B58" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>386</v>
+      </c>
+      <c r="D58" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E58" s="4"/>
+      <c r="F58" s="6"/>
+      <c r="G58" s="4" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7">
+      <c r="A59" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>389</v>
+      </c>
+      <c r="D59" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E59" s="4"/>
+      <c r="F59" s="6"/>
+      <c r="G59" s="4" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7">
+      <c r="A60" s="4" t="s">
+        <v>391</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C60" s="4" t="s">
         <v>392</v>
       </c>
+      <c r="D60" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E60" s="4"/>
+      <c r="F60" s="6"/>
+      <c r="G60" s="4" t="s">
+        <v>393</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:G47"/>
+  <autoFilter ref="A4:G60"/>
   <mergeCells count="2">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G3"/>

</xml_diff>